<commit_message>
Add condensed dashboard merging redundant KPIs (13 -> 9)
- New sheet '📊 لوحة مُكثّفة (٩ مؤشرات)' consolidating KPIs that serve the
  same objective, alongside the untouched original 13-KPI dashboard:
    * outage count   -> folded into fuel availability
    * inventory turnover -> folded into days-of-inventory (turnover = 30/days)
    * fill rate      -> removed (was a roll-up of stocked + PO timeliness)
    * accident count -> folded into safety/compliance rate
- Mirrors original styling: RTL, status conditional formatting, number formats
- Fix: COUNTIFS criteria ranges must match in size (orders sheet ends at row
  204, not 304) — caught by pycel verification
- Extend scripts/verify_formulas.py to cover both dashboards (14 cells, all pass)
- Add scripts/build_condensed_dashboard.py and document strategy in README

https://claude.ai/code/session_01KvBXTcUzJa33dDsqskcTMw
</commit_message>
<xml_diff>
--- a/workbook/khadija-supply-chain-kpis-2026.xlsx
+++ b/workbook/khadija-supply-chain-kpis-2026.xlsx
@@ -8,12 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="📊 ملخص آلي + KPIs" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="📋 مؤشرات الإدارة" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="🛢️ انقطاعات الوقود" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="💧 الردود والفاقد" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="📦 المخزون" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="🛒 الطلبات والمشتريات" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="🚚 النقل والرحلات" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="📊 لوحة مُكثّفة (٩ مؤشرات)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="📋 مؤشرات الإدارة" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="🛢️ انقطاعات الوقود" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="💧 الردود والفاقد" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="📦 المخزون" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="🛒 الطلبات والمشتريات" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="🚚 النقل والرحلات" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -30,7 +31,7 @@
     <numFmt numFmtId="168" formatCode="#,##0.0;\-#,##0.0;\-"/>
     <numFmt numFmtId="169" formatCode="yyyy\-mm\-dd\ hh:mm"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -184,8 +185,25 @@
       <color rgb="FF3D3D3D"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="DIN Next LT Arabic"/>
+      <b val="1"/>
+      <color rgb="FF3D3D3D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="DIN Next LT Arabic"/>
+      <b val="1"/>
+      <color rgb="FF1565C0"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="DIN Next LT Arabic"/>
+      <color rgb="FF1565C0"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -277,6 +295,11 @@
         <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF3741F"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -359,7 +382,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -644,6 +667,45 @@
     <xf numFmtId="169" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="25" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="22" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="25" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -653,7 +715,7 @@
     <cellStyle name="Currency [0]" xfId="4" builtinId="7"/>
     <cellStyle name="Percent" xfId="5" builtinId="5"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="6">
     <dxf>
       <font>
         <name val="DIN Next LT Arabic"/>
@@ -692,6 +754,36 @@
         <b val="1"/>
         <color rgb="FFC62828"/>
         <sz val="9"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEBEE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF2E7D32"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE8F5E9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFF9A825"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF8E1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC62828"/>
       </font>
       <fill>
         <patternFill>
@@ -2836,6 +2928,1312 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:R29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" style="40" min="1" max="1"/>
+    <col width="38" customWidth="1" style="40" min="2" max="2"/>
+    <col width="9" customWidth="1" style="40" min="3" max="3"/>
+    <col width="13" customWidth="1" style="40" min="4" max="4"/>
+    <col width="8" customWidth="1" style="40" min="5" max="5"/>
+    <col width="14" customWidth="1" style="40" min="6" max="6"/>
+    <col width="9" customWidth="1" style="40" min="7" max="7"/>
+    <col width="9" customWidth="1" style="40" min="8" max="8"/>
+    <col width="9" customWidth="1" style="40" min="9" max="9"/>
+    <col width="9" customWidth="1" style="40" min="10" max="10"/>
+    <col width="9" customWidth="1" style="40" min="11" max="11"/>
+    <col width="9" customWidth="1" style="40" min="12" max="12"/>
+    <col width="9" customWidth="1" style="40" min="13" max="13"/>
+    <col width="9" customWidth="1" style="40" min="14" max="14"/>
+    <col width="9" customWidth="1" style="40" min="15" max="15"/>
+    <col width="9" customWidth="1" style="40" min="16" max="16"/>
+    <col width="9" customWidth="1" style="40" min="17" max="17"/>
+    <col width="9" customWidth="1" style="40" min="18" max="18"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" s="40">
+      <c r="A1" s="96" t="inlineStr">
+        <is>
+          <t>📊 لوحة المؤشرات المُكثّفة — بعد دمج المتكرر (٩ مؤشرات)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="97" t="inlineStr">
+        <is>
+          <t>دُمج المتكرر: عدد الانقطاعات←التوفر · الدوران←أيام المخزون · Fill Rate (حُذف) · حوادث النقل←الامتثال/السلامة</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="98" t="inlineStr">
+        <is>
+          <t>📌 المؤشر</t>
+        </is>
+      </c>
+      <c r="G3" s="98" t="inlineStr">
+        <is>
+          <t>📅 الأشهر — خطة (يدوي) vs فعلي (آلي)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="99" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="99" t="inlineStr">
+        <is>
+          <t>المؤشر</t>
+        </is>
+      </c>
+      <c r="C4" s="99" t="inlineStr">
+        <is>
+          <t>الوحدة</t>
+        </is>
+      </c>
+      <c r="D4" s="99" t="inlineStr">
+        <is>
+          <t>الهدف</t>
+        </is>
+      </c>
+      <c r="E4" s="99" t="inlineStr">
+        <is>
+          <t>النوع</t>
+        </is>
+      </c>
+      <c r="F4" s="99" t="inlineStr">
+        <is>
+          <t>الانحراف</t>
+        </is>
+      </c>
+      <c r="G4" s="99" t="inlineStr">
+        <is>
+          <t>يناير</t>
+        </is>
+      </c>
+      <c r="H4" s="99" t="inlineStr">
+        <is>
+          <t>فبراير</t>
+        </is>
+      </c>
+      <c r="I4" s="99" t="inlineStr">
+        <is>
+          <t>مارس</t>
+        </is>
+      </c>
+      <c r="J4" s="99" t="inlineStr">
+        <is>
+          <t>أبريل</t>
+        </is>
+      </c>
+      <c r="K4" s="99" t="inlineStr">
+        <is>
+          <t>مايو</t>
+        </is>
+      </c>
+      <c r="L4" s="99" t="inlineStr">
+        <is>
+          <t>يونيو</t>
+        </is>
+      </c>
+      <c r="M4" s="99" t="inlineStr">
+        <is>
+          <t>يوليو</t>
+        </is>
+      </c>
+      <c r="N4" s="99" t="inlineStr">
+        <is>
+          <t>أغسطس</t>
+        </is>
+      </c>
+      <c r="O4" s="99" t="inlineStr">
+        <is>
+          <t>سبتمبر</t>
+        </is>
+      </c>
+      <c r="P4" s="99" t="inlineStr">
+        <is>
+          <t>أكتوبر</t>
+        </is>
+      </c>
+      <c r="Q4" s="99" t="inlineStr">
+        <is>
+          <t>نوفمبر</t>
+        </is>
+      </c>
+      <c r="R4" s="99" t="inlineStr">
+        <is>
+          <t>ديسمبر</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ◀ 👥 خدمة العميل</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="101" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="102" t="inlineStr">
+        <is>
+          <t>توفر الوقود (يطوي عدد الانقطاعات)</t>
+        </is>
+      </c>
+      <c r="C6" s="97" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D6" s="103" t="inlineStr">
+        <is>
+          <t>≥ 99.5%</t>
+        </is>
+      </c>
+      <c r="E6" s="97" t="inlineStr">
+        <is>
+          <t>خطة</t>
+        </is>
+      </c>
+      <c r="F6" s="97" t="n"/>
+      <c r="G6" s="104" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="H6" s="104" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="I6" s="104" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="J6" s="104" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="K6" s="104" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="L6" s="104" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="M6" s="104" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="N6" s="104" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="O6" s="104" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="P6" s="104" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="Q6" s="104" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="R6" s="104" t="n">
+        <v>0.995</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="E7" s="105" t="inlineStr">
+        <is>
+          <t>فعلي</t>
+        </is>
+      </c>
+      <c r="F7" s="105">
+        <f>IFERROR(IF(AVERAGE(G6:R6)=0,"",IF(IFERROR(AVERAGEIF(G7:R7,"&gt;0",G7:R7),0)&gt;=AVERAGE(G6:R6),"✅ ",IF(IFERROR(AVERAGEIF(G7:R7,"&gt;0",G7:R7),0)&gt;=AVERAGE(G6:R6)*0.85,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G7:R7,"&gt;0",G7:R7),0)-AVERAGE(G6:R6))/AVERAGE(G6:R6),"+0.0%;-0.0%")),"")</f>
+        <v/>
+      </c>
+      <c r="G7" s="106">
+        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,1,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,1+1,1))/('📊 ملخص آلي + KPIs'!$F$38*DAY(DATE(2026,1+1,1)-1))),1)</f>
+        <v/>
+      </c>
+      <c r="H7" s="106">
+        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,2,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,2+1,1))/('📊 ملخص آلي + KPIs'!$F$38*DAY(DATE(2026,2+1,1)-1))),1)</f>
+        <v/>
+      </c>
+      <c r="I7" s="106">
+        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,3,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,3+1,1))/('📊 ملخص آلي + KPIs'!$F$38*DAY(DATE(2026,3+1,1)-1))),1)</f>
+        <v/>
+      </c>
+      <c r="J7" s="106">
+        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,4,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,4+1,1))/('📊 ملخص آلي + KPIs'!$F$38*DAY(DATE(2026,4+1,1)-1))),1)</f>
+        <v/>
+      </c>
+      <c r="K7" s="106">
+        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,5,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,5+1,1))/('📊 ملخص آلي + KPIs'!$F$38*DAY(DATE(2026,5+1,1)-1))),1)</f>
+        <v/>
+      </c>
+      <c r="L7" s="106">
+        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,6,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,6+1,1))/('📊 ملخص آلي + KPIs'!$F$38*DAY(DATE(2026,6+1,1)-1))),1)</f>
+        <v/>
+      </c>
+      <c r="M7" s="106">
+        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,7,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,7+1,1))/('📊 ملخص آلي + KPIs'!$F$38*DAY(DATE(2026,7+1,1)-1))),1)</f>
+        <v/>
+      </c>
+      <c r="N7" s="106">
+        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,8,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,8+1,1))/('📊 ملخص آلي + KPIs'!$F$38*DAY(DATE(2026,8+1,1)-1))),1)</f>
+        <v/>
+      </c>
+      <c r="O7" s="106">
+        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,9,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,9+1,1))/('📊 ملخص آلي + KPIs'!$F$38*DAY(DATE(2026,9+1,1)-1))),1)</f>
+        <v/>
+      </c>
+      <c r="P7" s="106">
+        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,10,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,10+1,1))/('📊 ملخص آلي + KPIs'!$F$38*DAY(DATE(2026,10+1,1)-1))),1)</f>
+        <v/>
+      </c>
+      <c r="Q7" s="106">
+        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,11,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,11+1,1))/('📊 ملخص آلي + KPIs'!$F$38*DAY(DATE(2026,11+1,1)-1))),1)</f>
+        <v/>
+      </c>
+      <c r="R7" s="106">
+        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,12,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,12+1,1))/('📊 ملخص آلي + KPIs'!$F$38*DAY(DATE(2026,12+1,1)-1))),1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="101" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="102" t="inlineStr">
+        <is>
+          <t>توفر المواد المخزنية (تسليم ≤ 3 أيام)</t>
+        </is>
+      </c>
+      <c r="C8" s="97" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D8" s="103" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E8" s="97" t="inlineStr">
+        <is>
+          <t>خطة</t>
+        </is>
+      </c>
+      <c r="F8" s="97" t="n"/>
+      <c r="G8" s="104" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="104" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" s="104" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" s="104" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" s="104" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" s="104" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" s="104" t="n">
+        <v>1</v>
+      </c>
+      <c r="N8" s="104" t="n">
+        <v>1</v>
+      </c>
+      <c r="O8" s="104" t="n">
+        <v>1</v>
+      </c>
+      <c r="P8" s="104" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="104" t="n">
+        <v>1</v>
+      </c>
+      <c r="R8" s="104" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="E9" s="105" t="inlineStr">
+        <is>
+          <t>فعلي</t>
+        </is>
+      </c>
+      <c r="F9" s="105">
+        <f>IFERROR(IF(AVERAGE(G8:R8)=0,"",IF(IFERROR(AVERAGEIF(G9:R9,"&gt;0",G9:R9),0)&gt;=AVERAGE(G8:R8),"✅ ",IF(IFERROR(AVERAGEIF(G9:R9,"&gt;0",G9:R9),0)&gt;=AVERAGE(G8:R8)*0.85,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G9:R9,"&gt;0",G9:R9),0)-AVERAGE(G8:R8))/AVERAGE(G8:R8),"+0.0%;-0.0%")),"")</f>
+        <v/>
+      </c>
+      <c r="G9" s="106">
+        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,1,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,1+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,1,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,1+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
+        <v/>
+      </c>
+      <c r="H9" s="106">
+        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,2,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,2+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,2,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,2+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
+        <v/>
+      </c>
+      <c r="I9" s="106">
+        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,3,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,3+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,3,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,3+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
+        <v/>
+      </c>
+      <c r="J9" s="106">
+        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,4,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,4+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,4,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,4+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
+        <v/>
+      </c>
+      <c r="K9" s="106">
+        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,5,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,5+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,5,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,5+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
+        <v/>
+      </c>
+      <c r="L9" s="106">
+        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,6,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,6+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,6,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,6+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
+        <v/>
+      </c>
+      <c r="M9" s="106">
+        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,7,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,7+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,7,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,7+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
+        <v/>
+      </c>
+      <c r="N9" s="106">
+        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,8,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,8+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,8,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,8+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
+        <v/>
+      </c>
+      <c r="O9" s="106">
+        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,9,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,9+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,9,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,9+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
+        <v/>
+      </c>
+      <c r="P9" s="106">
+        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,10,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,10+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,10,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,10+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
+        <v/>
+      </c>
+      <c r="Q9" s="106">
+        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,11,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,11+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,11,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,11+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
+        <v/>
+      </c>
+      <c r="R9" s="106">
+        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,12,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,12+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,12,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,12+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="101" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" s="102" t="inlineStr">
+        <is>
+          <t>إصدار أوامر الشراء (≤ 5 أيام عمل)</t>
+        </is>
+      </c>
+      <c r="C10" s="97" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D10" s="103" t="inlineStr">
+        <is>
+          <t>≥ 95%</t>
+        </is>
+      </c>
+      <c r="E10" s="97" t="inlineStr">
+        <is>
+          <t>خطة</t>
+        </is>
+      </c>
+      <c r="F10" s="97" t="n"/>
+      <c r="G10" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H10" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="I10" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J10" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="K10" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L10" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="M10" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="N10" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="O10" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="P10" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="Q10" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="R10" s="104" t="n">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="E11" s="105" t="inlineStr">
+        <is>
+          <t>فعلي</t>
+        </is>
+      </c>
+      <c r="F11" s="105">
+        <f>IFERROR(IF(AVERAGE(G10:R10)=0,"",IF(IFERROR(AVERAGEIF(G11:R11,"&gt;0",G11:R11),0)&gt;=AVERAGE(G10:R10),"✅ ",IF(IFERROR(AVERAGEIF(G11:R11,"&gt;0",G11:R11),0)&gt;=AVERAGE(G10:R10)*0.85,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G11:R11,"&gt;0",G11:R11),0)-AVERAGE(G10:R10))/AVERAGE(G10:R10),"+0.0%;-0.0%")),"")</f>
+        <v/>
+      </c>
+      <c r="G11" s="106">
+        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,1,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,1+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,1,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,1+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
+        <v/>
+      </c>
+      <c r="H11" s="106">
+        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,2,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,2+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,2,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,2+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
+        <v/>
+      </c>
+      <c r="I11" s="106">
+        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,3,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,3+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,3,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,3+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
+        <v/>
+      </c>
+      <c r="J11" s="106">
+        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,4,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,4+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,4,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,4+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
+        <v/>
+      </c>
+      <c r="K11" s="106">
+        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,5,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,5+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,5,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,5+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
+        <v/>
+      </c>
+      <c r="L11" s="106">
+        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,6,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,6+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,6,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,6+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
+        <v/>
+      </c>
+      <c r="M11" s="106">
+        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,7,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,7+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,7,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,7+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
+        <v/>
+      </c>
+      <c r="N11" s="106">
+        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,8,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,8+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,8,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,8+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
+        <v/>
+      </c>
+      <c r="O11" s="106">
+        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,9,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,9+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,9,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,9+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
+        <v/>
+      </c>
+      <c r="P11" s="106">
+        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,10,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,10+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,10,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,10+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
+        <v/>
+      </c>
+      <c r="Q11" s="106">
+        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,11,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,11+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,11,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,11+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
+        <v/>
+      </c>
+      <c r="R11" s="106">
+        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,12,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,12+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,12,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,12+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ◀ 💰 التكاليف</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="101" t="n">
+        <v>4</v>
+      </c>
+      <c r="B13" s="102" t="inlineStr">
+        <is>
+          <t>فواقد الوقود لكل 33K لتر</t>
+        </is>
+      </c>
+      <c r="C13" s="97" t="inlineStr">
+        <is>
+          <t>لتر</t>
+        </is>
+      </c>
+      <c r="D13" s="103" t="inlineStr">
+        <is>
+          <t>≤ 100</t>
+        </is>
+      </c>
+      <c r="E13" s="97" t="inlineStr">
+        <is>
+          <t>خطة</t>
+        </is>
+      </c>
+      <c r="F13" s="97" t="n"/>
+      <c r="G13" s="107" t="n">
+        <v>100</v>
+      </c>
+      <c r="H13" s="107" t="n">
+        <v>100</v>
+      </c>
+      <c r="I13" s="107" t="n">
+        <v>100</v>
+      </c>
+      <c r="J13" s="107" t="n">
+        <v>100</v>
+      </c>
+      <c r="K13" s="107" t="n">
+        <v>100</v>
+      </c>
+      <c r="L13" s="107" t="n">
+        <v>100</v>
+      </c>
+      <c r="M13" s="107" t="n">
+        <v>100</v>
+      </c>
+      <c r="N13" s="107" t="n">
+        <v>100</v>
+      </c>
+      <c r="O13" s="107" t="n">
+        <v>100</v>
+      </c>
+      <c r="P13" s="107" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q13" s="107" t="n">
+        <v>100</v>
+      </c>
+      <c r="R13" s="107" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="E14" s="105" t="inlineStr">
+        <is>
+          <t>فعلي</t>
+        </is>
+      </c>
+      <c r="F14" s="105">
+        <f>IFERROR(IF(AVERAGE(G13:R13)=0,"",IF(IFERROR(AVERAGEIF(G14:R14,"&gt;0",G14:R14),0)&lt;=AVERAGE(G13:R13),"✅ ",IF(IFERROR(AVERAGEIF(G14:R14,"&gt;0",G14:R14),0)&lt;=AVERAGE(G13:R13)*1.3,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G14:R14,"&gt;0",G14:R14),0)-AVERAGE(G13:R13))/AVERAGE(G13:R13),"+0.0%;-0.0%")),"")</f>
+        <v/>
+      </c>
+      <c r="G14" s="108">
+        <f>IFERROR(SUMIFS('💧 الردود والفاقد'!G5:G304,'💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,1,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,1+1,1))/COUNTIFS('💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,1,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,1+1,1)),0)</f>
+        <v/>
+      </c>
+      <c r="H14" s="108">
+        <f>IFERROR(SUMIFS('💧 الردود والفاقد'!G5:G304,'💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,2,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,2+1,1))/COUNTIFS('💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,2,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,2+1,1)),0)</f>
+        <v/>
+      </c>
+      <c r="I14" s="108">
+        <f>IFERROR(SUMIFS('💧 الردود والفاقد'!G5:G304,'💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,3,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,3+1,1))/COUNTIFS('💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,3,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,3+1,1)),0)</f>
+        <v/>
+      </c>
+      <c r="J14" s="108">
+        <f>IFERROR(SUMIFS('💧 الردود والفاقد'!G5:G304,'💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,4,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,4+1,1))/COUNTIFS('💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,4,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,4+1,1)),0)</f>
+        <v/>
+      </c>
+      <c r="K14" s="108">
+        <f>IFERROR(SUMIFS('💧 الردود والفاقد'!G5:G304,'💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,5,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,5+1,1))/COUNTIFS('💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,5,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,5+1,1)),0)</f>
+        <v/>
+      </c>
+      <c r="L14" s="108">
+        <f>IFERROR(SUMIFS('💧 الردود والفاقد'!G5:G304,'💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,6,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,6+1,1))/COUNTIFS('💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,6,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,6+1,1)),0)</f>
+        <v/>
+      </c>
+      <c r="M14" s="108">
+        <f>IFERROR(SUMIFS('💧 الردود والفاقد'!G5:G304,'💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,7,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,7+1,1))/COUNTIFS('💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,7,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,7+1,1)),0)</f>
+        <v/>
+      </c>
+      <c r="N14" s="108">
+        <f>IFERROR(SUMIFS('💧 الردود والفاقد'!G5:G304,'💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,8,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,8+1,1))/COUNTIFS('💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,8,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,8+1,1)),0)</f>
+        <v/>
+      </c>
+      <c r="O14" s="108">
+        <f>IFERROR(SUMIFS('💧 الردود والفاقد'!G5:G304,'💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,9,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,9+1,1))/COUNTIFS('💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,9,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,9+1,1)),0)</f>
+        <v/>
+      </c>
+      <c r="P14" s="108">
+        <f>IFERROR(SUMIFS('💧 الردود والفاقد'!G5:G304,'💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,10,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,10+1,1))/COUNTIFS('💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,10,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,10+1,1)),0)</f>
+        <v/>
+      </c>
+      <c r="Q14" s="108">
+        <f>IFERROR(SUMIFS('💧 الردود والفاقد'!G5:G304,'💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,11,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,11+1,1))/COUNTIFS('💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,11,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,11+1,1)),0)</f>
+        <v/>
+      </c>
+      <c r="R14" s="108">
+        <f>IFERROR(SUMIFS('💧 الردود والفاقد'!G5:G304,'💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,12,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,12+1,1))/COUNTIFS('💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,12,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,12+1,1)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="101" t="n">
+        <v>5</v>
+      </c>
+      <c r="B15" s="102" t="inlineStr">
+        <is>
+          <t>نسبة المواد التالفة (يدوي شهرياً)</t>
+        </is>
+      </c>
+      <c r="C15" s="97" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D15" s="103" t="inlineStr">
+        <is>
+          <t>≤ 2%</t>
+        </is>
+      </c>
+      <c r="E15" s="97" t="inlineStr">
+        <is>
+          <t>خطة</t>
+        </is>
+      </c>
+      <c r="F15" s="97" t="n"/>
+      <c r="G15" s="104" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="H15" s="104" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="I15" s="104" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="J15" s="104" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="K15" s="104" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="L15" s="104" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="M15" s="104" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="N15" s="104" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="O15" s="104" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="P15" s="104" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="Q15" s="104" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="R15" s="104" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="E16" s="105" t="inlineStr">
+        <is>
+          <t>فعلي</t>
+        </is>
+      </c>
+      <c r="F16" s="105">
+        <f>IFERROR(IF(AVERAGE(G15:R15)=0,"",IF(IFERROR(AVERAGEIF(G16:R16,"&gt;0",G16:R16),0)&lt;=AVERAGE(G15:R15),"✅ ",IF(IFERROR(AVERAGEIF(G16:R16,"&gt;0",G16:R16),0)&lt;=AVERAGE(G15:R15)*1.3,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G16:R16,"&gt;0",G16:R16),0)-AVERAGE(G15:R15))/AVERAGE(G15:R15),"+0.0%;-0.0%")),"")</f>
+        <v/>
+      </c>
+      <c r="G16" s="106" t="n"/>
+      <c r="H16" s="106" t="n"/>
+      <c r="I16" s="106" t="n"/>
+      <c r="J16" s="106" t="n"/>
+      <c r="K16" s="106" t="n"/>
+      <c r="L16" s="106" t="n"/>
+      <c r="M16" s="106" t="n"/>
+      <c r="N16" s="106" t="n"/>
+      <c r="O16" s="106" t="n"/>
+      <c r="P16" s="106" t="n"/>
+      <c r="Q16" s="106" t="n"/>
+      <c r="R16" s="106" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ◀ 🏦 السيولة المالية</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="101" t="n">
+        <v>6</v>
+      </c>
+      <c r="B18" s="102" t="inlineStr">
+        <is>
+          <t>أيام مخزون الوقود (يطوي الدوران)</t>
+        </is>
+      </c>
+      <c r="C18" s="97" t="inlineStr">
+        <is>
+          <t>يوم</t>
+        </is>
+      </c>
+      <c r="D18" s="103" t="inlineStr">
+        <is>
+          <t>≤ 3</t>
+        </is>
+      </c>
+      <c r="E18" s="97" t="inlineStr">
+        <is>
+          <t>خطة</t>
+        </is>
+      </c>
+      <c r="F18" s="97" t="n"/>
+      <c r="G18" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="H18" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="I18" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="J18" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="K18" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="L18" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="M18" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="N18" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="O18" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="P18" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q18" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="R18" s="107" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="E19" s="105" t="inlineStr">
+        <is>
+          <t>فعلي</t>
+        </is>
+      </c>
+      <c r="F19" s="105">
+        <f>IFERROR(IF(AVERAGE(G18:R18)=0,"",IF(IFERROR(AVERAGEIF(G19:R19,"&gt;0",G19:R19),0)&lt;=AVERAGE(G18:R18),"✅ ",IF(IFERROR(AVERAGEIF(G19:R19,"&gt;0",G19:R19),0)&lt;=AVERAGE(G18:R18)*1.3,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G19:R19,"&gt;0",G19:R19),0)-AVERAGE(G18:R18))/AVERAGE(G18:R18),"+0.0%;-0.0%")),"")</f>
+        <v/>
+      </c>
+      <c r="G19" s="108">
+        <f>IFERROR(AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,1,'📦 المخزون'!F5:F304,"وقود"),0)</f>
+        <v/>
+      </c>
+      <c r="H19" s="108">
+        <f>IFERROR(AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,2,'📦 المخزون'!F5:F304,"وقود"),0)</f>
+        <v/>
+      </c>
+      <c r="I19" s="108">
+        <f>IFERROR(AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,3,'📦 المخزون'!F5:F304,"وقود"),0)</f>
+        <v/>
+      </c>
+      <c r="J19" s="108">
+        <f>IFERROR(AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,4,'📦 المخزون'!F5:F304,"وقود"),0)</f>
+        <v/>
+      </c>
+      <c r="K19" s="108">
+        <f>IFERROR(AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,5,'📦 المخزون'!F5:F304,"وقود"),0)</f>
+        <v/>
+      </c>
+      <c r="L19" s="108">
+        <f>IFERROR(AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,6,'📦 المخزون'!F5:F304,"وقود"),0)</f>
+        <v/>
+      </c>
+      <c r="M19" s="108">
+        <f>IFERROR(AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,7,'📦 المخزون'!F5:F304,"وقود"),0)</f>
+        <v/>
+      </c>
+      <c r="N19" s="108">
+        <f>IFERROR(AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,8,'📦 المخزون'!F5:F304,"وقود"),0)</f>
+        <v/>
+      </c>
+      <c r="O19" s="108">
+        <f>IFERROR(AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,9,'📦 المخزون'!F5:F304,"وقود"),0)</f>
+        <v/>
+      </c>
+      <c r="P19" s="108">
+        <f>IFERROR(AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,10,'📦 المخزون'!F5:F304,"وقود"),0)</f>
+        <v/>
+      </c>
+      <c r="Q19" s="108">
+        <f>IFERROR(AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,11,'📦 المخزون'!F5:F304,"وقود"),0)</f>
+        <v/>
+      </c>
+      <c r="R19" s="108">
+        <f>IFERROR(AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,12,'📦 المخزون'!F5:F304,"وقود"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ◀ 🛡️ السلامة والامتثال</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="101" t="n">
+        <v>7</v>
+      </c>
+      <c r="B21" s="102" t="inlineStr">
+        <is>
+          <t>الامتثال والسلامة (يطوي عدد الحوادث)</t>
+        </is>
+      </c>
+      <c r="C21" s="97" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D21" s="103" t="inlineStr">
+        <is>
+          <t>≥ 95%</t>
+        </is>
+      </c>
+      <c r="E21" s="97" t="inlineStr">
+        <is>
+          <t>خطة</t>
+        </is>
+      </c>
+      <c r="F21" s="97" t="n"/>
+      <c r="G21" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H21" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="I21" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J21" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="K21" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L21" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="M21" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="N21" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="O21" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="P21" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="Q21" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="R21" s="104" t="n">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="E22" s="105" t="inlineStr">
+        <is>
+          <t>فعلي</t>
+        </is>
+      </c>
+      <c r="F22" s="105">
+        <f>IFERROR(IF(AVERAGE(G21:R21)=0,"",IF(IFERROR(AVERAGEIF(G22:R22,"&gt;0",G22:R22),0)&gt;=AVERAGE(G21:R21),"✅ ",IF(IFERROR(AVERAGEIF(G22:R22,"&gt;0",G22:R22),0)&gt;=AVERAGE(G21:R21)*0.85,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G22:R22,"&gt;0",G22:R22),0)-AVERAGE(G21:R21))/AVERAGE(G21:R21),"+0.0%;-0.0%")),"")</f>
+        <v/>
+      </c>
+      <c r="G22" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,1,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,1+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,1,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,1+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="H22" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,2,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,2+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,2,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,2+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="I22" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,3,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,3+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,3,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,3+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="J22" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,4,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,4+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,4,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,4+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="K22" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,5,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,5+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,5,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,5+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="L22" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,6,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,6+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,6,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,6+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="M22" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,7,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,7+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,7,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,7+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="N22" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,8,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,8+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,8,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,8+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="O22" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,9,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,9+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,9,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,9+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="P22" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,10,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,10+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,10,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,10+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="Q22" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,11,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,11+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,11,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,11+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="R22" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,12,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,12+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,12,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,12+1,1))),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ◀ ⚙️ الكفاءة التشغيلية</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="101" t="n">
+        <v>8</v>
+      </c>
+      <c r="B24" s="102" t="inlineStr">
+        <is>
+          <t>التزام جدول النقل (On-time)</t>
+        </is>
+      </c>
+      <c r="C24" s="97" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D24" s="103" t="inlineStr">
+        <is>
+          <t>≥ 95%</t>
+        </is>
+      </c>
+      <c r="E24" s="97" t="inlineStr">
+        <is>
+          <t>خطة</t>
+        </is>
+      </c>
+      <c r="F24" s="97" t="n"/>
+      <c r="G24" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H24" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="I24" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J24" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="K24" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L24" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="M24" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="N24" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="O24" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="P24" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="Q24" s="104" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="R24" s="104" t="n">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="E25" s="105" t="inlineStr">
+        <is>
+          <t>فعلي</t>
+        </is>
+      </c>
+      <c r="F25" s="105">
+        <f>IFERROR(IF(AVERAGE(G24:R24)=0,"",IF(IFERROR(AVERAGEIF(G25:R25,"&gt;0",G25:R25),0)&gt;=AVERAGE(G24:R24),"✅ ",IF(IFERROR(AVERAGEIF(G25:R25,"&gt;0",G25:R25),0)&gt;=AVERAGE(G24:R24)*0.85,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G25:R25,"&gt;0",G25:R25),0)-AVERAGE(G24:R24))/AVERAGE(G24:R24),"+0.0%;-0.0%")),"")</f>
+        <v/>
+      </c>
+      <c r="G25" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,1,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,1+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,1,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,1+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="H25" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,2,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,2+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,2,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,2+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="I25" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,3,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,3+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,3,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,3+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="J25" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,4,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,4+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,4,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,4+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="K25" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,5,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,5+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,5,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,5+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="L25" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,6,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,6+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,6,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,6+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="M25" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,7,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,7+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,7,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,7+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="N25" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,8,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,8+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,8,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,8+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="O25" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,9,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,9+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,9,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,9+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="P25" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,10,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,10+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,10,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,10+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="Q25" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,11,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,11+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,11,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,11+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="R25" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,12,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,12+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,12,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,12+1,1))),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="101" t="n">
+        <v>9</v>
+      </c>
+      <c r="B26" s="102" t="inlineStr">
+        <is>
+          <t>نسبة استخدام الأسطول المملوك</t>
+        </is>
+      </c>
+      <c r="C26" s="97" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D26" s="103" t="inlineStr">
+        <is>
+          <t>≥ 60%</t>
+        </is>
+      </c>
+      <c r="E26" s="97" t="inlineStr">
+        <is>
+          <t>خطة</t>
+        </is>
+      </c>
+      <c r="F26" s="97" t="n"/>
+      <c r="G26" s="104" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H26" s="104" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I26" s="104" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J26" s="104" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="K26" s="104" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L26" s="104" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="M26" s="104" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="N26" s="104" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="O26" s="104" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="P26" s="104" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="Q26" s="104" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="R26" s="104" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="E27" s="105" t="inlineStr">
+        <is>
+          <t>فعلي</t>
+        </is>
+      </c>
+      <c r="F27" s="105">
+        <f>IFERROR(IF(AVERAGE(G26:R26)=0,"",IF(IFERROR(AVERAGEIF(G27:R27,"&gt;0",G27:R27),0)&gt;=AVERAGE(G26:R26),"✅ ",IF(IFERROR(AVERAGEIF(G27:R27,"&gt;0",G27:R27),0)&gt;=AVERAGE(G26:R26)*0.85,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G27:R27,"&gt;0",G27:R27),0)-AVERAGE(G26:R26))/AVERAGE(G26:R26),"+0.0%;-0.0%")),"")</f>
+        <v/>
+      </c>
+      <c r="G27" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,1,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,1+1,1),'🚚 النقل والرحلات'!G5:G304,"مملوك درب")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,1,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,1+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="H27" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,2,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,2+1,1),'🚚 النقل والرحلات'!G5:G304,"مملوك درب")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,2,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,2+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="I27" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,3,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,3+1,1),'🚚 النقل والرحلات'!G5:G304,"مملوك درب")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,3,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,3+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="J27" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,4,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,4+1,1),'🚚 النقل والرحلات'!G5:G304,"مملوك درب")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,4,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,4+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="K27" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,5,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,5+1,1),'🚚 النقل والرحلات'!G5:G304,"مملوك درب")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,5,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,5+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="L27" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,6,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,6+1,1),'🚚 النقل والرحلات'!G5:G304,"مملوك درب")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,6,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,6+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="M27" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,7,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,7+1,1),'🚚 النقل والرحلات'!G5:G304,"مملوك درب")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,7,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,7+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="N27" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,8,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,8+1,1),'🚚 النقل والرحلات'!G5:G304,"مملوك درب")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,8,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,8+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="O27" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,9,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,9+1,1),'🚚 النقل والرحلات'!G5:G304,"مملوك درب")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,9,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,9+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="P27" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,10,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,10+1,1),'🚚 النقل والرحلات'!G5:G304,"مملوك درب")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,10,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,10+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="Q27" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,11,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,11+1,1),'🚚 النقل والرحلات'!G5:G304,"مملوك درب")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,11,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,11+1,1))),0)</f>
+        <v/>
+      </c>
+      <c r="R27" s="106">
+        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,12,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,12+1,1),'🚚 النقل والرحلات'!G5:G304,"مملوك درب")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,12,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,12+1,1))),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="83" t="inlineStr">
+        <is>
+          <t>ℹ️ المقاييس المطوية متاحة كتشخيص في اللوحة الأصلية: عدد الانقطاعات، دوران المخزون، عدد الحوادث الجسيمة، ونسبة استيفاء الطلبات (Fill Rate).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="46">
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="G3:R3"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="A12:R12"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="A5:R5"/>
+    <mergeCell ref="A17:R17"/>
+    <mergeCell ref="A23:R23"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="A20:R20"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A29:R29"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="B21:B22"/>
+  </mergeCells>
+  <conditionalFormatting sqref="F6:F28">
+    <cfRule type="expression" priority="1" dxfId="3">
+      <formula>ISNUMBER(SEARCH("✅",F6))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="4">
+      <formula>ISNUMBER(SEARCH("🟡",F6))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="5">
+      <formula>ISNUMBER(SEARCH("🔴",F6))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3118,7 +4516,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4731,7 +6129,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10554,7 +11952,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -17589,7 +18987,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -21518,7 +22916,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add per-axis roll-up status and numeric target column
- Condensed dashboard: each axis header now shows a roll-up status in column F
  (worst status among its KPIs), auto-colored by the same conditional formatting
- Both dashboards: 'الهدف' (target) column is now a real number (e.g. 99.50%, 100, 3)
  matching the plan-cell format, instead of text like '≥ 99.5%'
- Extend verification to 19 cells (incl. 5 axis roll-ups); fix verify comparison
  to handle string (emoji) expectations
- Preserves RTL, conditional formatting, dropdowns; document in README

https://claude.ai/code/session_01KvBXTcUzJa33dDsqskcTMw
</commit_message>
<xml_diff>
--- a/workbook/khadija-supply-chain-kpis-2026.xlsx
+++ b/workbook/khadija-supply-chain-kpis-2026.xlsx
@@ -31,7 +31,7 @@
     <numFmt numFmtId="168" formatCode="#,##0.0;\-#,##0.0;\-"/>
     <numFmt numFmtId="169" formatCode="yyyy\-mm\-dd\ hh:mm"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="27">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -201,6 +201,12 @@
       <name val="DIN Next LT Arabic"/>
       <color rgb="FF1565C0"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="DIN Next LT Arabic"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="18">
@@ -382,7 +388,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="117">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -704,6 +710,30 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="22" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="11" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="24" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="24" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1187,10 +1217,8 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D6" s="50" t="inlineStr">
-        <is>
-          <t>≥ 99.5%</t>
-        </is>
+      <c r="D6" s="109" t="n">
+        <v>0.995</v>
       </c>
       <c r="E6" s="51" t="inlineStr">
         <is>
@@ -1312,10 +1340,8 @@
           <t>انقطاع</t>
         </is>
       </c>
-      <c r="D8" s="50" t="inlineStr">
-        <is>
-          <t>≤ 5</t>
-        </is>
+      <c r="D8" s="110" t="n">
+        <v>5</v>
       </c>
       <c r="E8" s="51" t="inlineStr">
         <is>
@@ -1437,10 +1463,8 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D10" s="50" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
+      <c r="D10" s="111" t="n">
+        <v>1</v>
       </c>
       <c r="E10" s="51" t="inlineStr">
         <is>
@@ -1562,10 +1586,8 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D12" s="50" t="inlineStr">
-        <is>
-          <t>≥ 95%</t>
-        </is>
+      <c r="D12" s="111" t="n">
+        <v>0.95</v>
       </c>
       <c r="E12" s="51" t="inlineStr">
         <is>
@@ -1687,10 +1709,8 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D14" s="50" t="inlineStr">
-        <is>
-          <t>≥ 98%</t>
-        </is>
+      <c r="D14" s="111" t="n">
+        <v>0.98</v>
       </c>
       <c r="E14" s="51" t="inlineStr">
         <is>
@@ -1819,10 +1839,8 @@
           <t>لتر</t>
         </is>
       </c>
-      <c r="D17" s="50" t="inlineStr">
-        <is>
-          <t>≤ 100</t>
-        </is>
+      <c r="D17" s="112" t="n">
+        <v>100</v>
       </c>
       <c r="E17" s="51" t="inlineStr">
         <is>
@@ -1944,10 +1962,8 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D19" s="50" t="inlineStr">
-        <is>
-          <t>≤ 2%</t>
-        </is>
+      <c r="D19" s="111" t="n">
+        <v>0.02</v>
       </c>
       <c r="E19" s="51" t="inlineStr">
         <is>
@@ -2064,10 +2080,8 @@
           <t>يوم</t>
         </is>
       </c>
-      <c r="D22" s="50" t="inlineStr">
-        <is>
-          <t>≤ 3</t>
-        </is>
+      <c r="D22" s="112" t="n">
+        <v>3</v>
       </c>
       <c r="E22" s="51" t="inlineStr">
         <is>
@@ -2189,10 +2203,8 @@
           <t>مرة</t>
         </is>
       </c>
-      <c r="D24" s="50" t="inlineStr">
-        <is>
-          <t>≥ 10</t>
-        </is>
+      <c r="D24" s="112" t="n">
+        <v>10</v>
       </c>
       <c r="E24" s="51" t="inlineStr">
         <is>
@@ -2321,10 +2333,8 @@
           <t>حادث</t>
         </is>
       </c>
-      <c r="D27" s="50" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D27" s="110" t="n">
+        <v>0</v>
       </c>
       <c r="E27" s="51" t="inlineStr">
         <is>
@@ -2446,10 +2456,8 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D29" s="50" t="inlineStr">
-        <is>
-          <t>≥ 95%</t>
-        </is>
+      <c r="D29" s="111" t="n">
+        <v>0.95</v>
       </c>
       <c r="E29" s="51" t="inlineStr">
         <is>
@@ -2578,10 +2586,8 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D32" s="50" t="inlineStr">
-        <is>
-          <t>≥ 95%</t>
-        </is>
+      <c r="D32" s="111" t="n">
+        <v>0.95</v>
       </c>
       <c r="E32" s="51" t="inlineStr">
         <is>
@@ -2703,10 +2709,8 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D34" s="50" t="inlineStr">
-        <is>
-          <t>≥ 60%</t>
-        </is>
+      <c r="D34" s="111" t="n">
+        <v>0.6</v>
       </c>
       <c r="E34" s="51" t="inlineStr">
         <is>
@@ -3075,6 +3079,11 @@
           <t xml:space="preserve">  ◀ 👥 خدمة العميل</t>
         </is>
       </c>
+      <c r="F5" s="113">
+        <f>IF(COUNTIF(F6:F11,"*🔴*")&gt;0,"🔴",IF(COUNTIF(F6:F11,"*🟡*")&gt;0,"🟡","✅"))</f>
+        <v/>
+      </c>
+      <c r="G5" s="114" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="101" t="n">
@@ -3090,10 +3099,8 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D6" s="103" t="inlineStr">
-        <is>
-          <t>≥ 99.5%</t>
-        </is>
+      <c r="D6" s="115" t="n">
+        <v>0.995</v>
       </c>
       <c r="E6" s="97" t="inlineStr">
         <is>
@@ -3211,10 +3218,8 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D8" s="103" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
+      <c r="D8" s="115" t="n">
+        <v>1</v>
       </c>
       <c r="E8" s="97" t="inlineStr">
         <is>
@@ -3332,10 +3337,8 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D10" s="103" t="inlineStr">
-        <is>
-          <t>≥ 95%</t>
-        </is>
+      <c r="D10" s="115" t="n">
+        <v>0.95</v>
       </c>
       <c r="E10" s="97" t="inlineStr">
         <is>
@@ -3445,6 +3448,11 @@
           <t xml:space="preserve">  ◀ 💰 التكاليف</t>
         </is>
       </c>
+      <c r="F12" s="113">
+        <f>IF(COUNTIF(F13:F16,"*🔴*")&gt;0,"🔴",IF(COUNTIF(F13:F16,"*🟡*")&gt;0,"🟡","✅"))</f>
+        <v/>
+      </c>
+      <c r="G12" s="114" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="101" t="n">
@@ -3460,10 +3468,8 @@
           <t>لتر</t>
         </is>
       </c>
-      <c r="D13" s="103" t="inlineStr">
-        <is>
-          <t>≤ 100</t>
-        </is>
+      <c r="D13" s="116" t="n">
+        <v>100</v>
       </c>
       <c r="E13" s="97" t="inlineStr">
         <is>
@@ -3581,10 +3587,8 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D15" s="103" t="inlineStr">
-        <is>
-          <t>≤ 2%</t>
-        </is>
+      <c r="D15" s="115" t="n">
+        <v>0.02</v>
       </c>
       <c r="E15" s="97" t="inlineStr">
         <is>
@@ -3658,6 +3662,11 @@
           <t xml:space="preserve">  ◀ 🏦 السيولة المالية</t>
         </is>
       </c>
+      <c r="F17" s="113">
+        <f>IF(COUNTIF(F18:F19,"*🔴*")&gt;0,"🔴",IF(COUNTIF(F18:F19,"*🟡*")&gt;0,"🟡","✅"))</f>
+        <v/>
+      </c>
+      <c r="G17" s="114" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="101" t="n">
@@ -3673,10 +3682,8 @@
           <t>يوم</t>
         </is>
       </c>
-      <c r="D18" s="103" t="inlineStr">
-        <is>
-          <t>≤ 3</t>
-        </is>
+      <c r="D18" s="116" t="n">
+        <v>3</v>
       </c>
       <c r="E18" s="97" t="inlineStr">
         <is>
@@ -3786,6 +3793,11 @@
           <t xml:space="preserve">  ◀ 🛡️ السلامة والامتثال</t>
         </is>
       </c>
+      <c r="F20" s="113">
+        <f>IF(COUNTIF(F21:F22,"*🔴*")&gt;0,"🔴",IF(COUNTIF(F21:F22,"*🟡*")&gt;0,"🟡","✅"))</f>
+        <v/>
+      </c>
+      <c r="G20" s="114" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="101" t="n">
@@ -3801,10 +3813,8 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D21" s="103" t="inlineStr">
-        <is>
-          <t>≥ 95%</t>
-        </is>
+      <c r="D21" s="115" t="n">
+        <v>0.95</v>
       </c>
       <c r="E21" s="97" t="inlineStr">
         <is>
@@ -3914,6 +3924,11 @@
           <t xml:space="preserve">  ◀ ⚙️ الكفاءة التشغيلية</t>
         </is>
       </c>
+      <c r="F23" s="113">
+        <f>IF(COUNTIF(F24:F27,"*🔴*")&gt;0,"🔴",IF(COUNTIF(F24:F27,"*🟡*")&gt;0,"🟡","✅"))</f>
+        <v/>
+      </c>
+      <c r="G23" s="114" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="101" t="n">
@@ -3929,10 +3944,8 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D24" s="103" t="inlineStr">
-        <is>
-          <t>≥ 95%</t>
-        </is>
+      <c r="D24" s="115" t="n">
+        <v>0.95</v>
       </c>
       <c r="E24" s="97" t="inlineStr">
         <is>
@@ -4050,10 +4063,8 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D26" s="103" t="inlineStr">
-        <is>
-          <t>≥ 60%</t>
-        </is>
+      <c r="D26" s="115" t="n">
+        <v>0.6</v>
       </c>
       <c r="E26" s="97" t="inlineStr">
         <is>
@@ -4165,7 +4176,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="46">
+  <mergeCells count="51">
     <mergeCell ref="A24:A25"/>
     <mergeCell ref="B18:B19"/>
     <mergeCell ref="D21:D22"/>
@@ -4175,16 +4186,13 @@
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="G3:R3"/>
     <mergeCell ref="C26:C27"/>
-    <mergeCell ref="A12:R12"/>
     <mergeCell ref="B26:B27"/>
     <mergeCell ref="A2:R2"/>
     <mergeCell ref="B13:B14"/>
     <mergeCell ref="A26:A27"/>
     <mergeCell ref="D13:D14"/>
+    <mergeCell ref="G5:R5"/>
     <mergeCell ref="C21:C22"/>
-    <mergeCell ref="A5:R5"/>
-    <mergeCell ref="A17:R17"/>
-    <mergeCell ref="A23:R23"/>
     <mergeCell ref="B10:B11"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A18:A19"/>
@@ -4193,35 +4201,43 @@
     <mergeCell ref="A21:A22"/>
     <mergeCell ref="D24:D25"/>
     <mergeCell ref="D15:D16"/>
-    <mergeCell ref="A20:R20"/>
+    <mergeCell ref="G20:R20"/>
+    <mergeCell ref="A12:E12"/>
     <mergeCell ref="A8:A9"/>
     <mergeCell ref="A29:R29"/>
     <mergeCell ref="C8:C9"/>
     <mergeCell ref="D18:D19"/>
     <mergeCell ref="A13:A14"/>
     <mergeCell ref="D8:D9"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A23:E23"/>
     <mergeCell ref="C18:C19"/>
     <mergeCell ref="A10:A11"/>
+    <mergeCell ref="A17:E17"/>
     <mergeCell ref="C13:C14"/>
+    <mergeCell ref="G12:R12"/>
     <mergeCell ref="D10:D11"/>
+    <mergeCell ref="A20:E20"/>
     <mergeCell ref="D26:D27"/>
     <mergeCell ref="A15:A16"/>
     <mergeCell ref="C15:C16"/>
+    <mergeCell ref="G23:R23"/>
     <mergeCell ref="A1:R1"/>
     <mergeCell ref="C6:C7"/>
     <mergeCell ref="C24:C25"/>
     <mergeCell ref="D6:D7"/>
+    <mergeCell ref="G17:R17"/>
     <mergeCell ref="B21:B22"/>
   </mergeCells>
-  <conditionalFormatting sqref="F6:F28">
+  <conditionalFormatting sqref="F5:F28">
     <cfRule type="expression" priority="1" dxfId="3">
-      <formula>ISNUMBER(SEARCH("✅",F6))</formula>
+      <formula>ISNUMBER(SEARCH("✅",F5))</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="4">
-      <formula>ISNUMBER(SEARCH("🟡",F6))</formula>
+      <formula>ISNUMBER(SEARCH("🟡",F5))</formula>
     </cfRule>
     <cfRule type="expression" priority="3" dxfId="5">
-      <formula>ISNUMBER(SEARCH("🔴",F6))</formula>
+      <formula>ISNUMBER(SEARCH("🔴",F5))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Consolidate to a single 9-KPI dashboard (remove the 13-KPI sheet)
- Build '📊 مؤشرات الأداء (٩)' as the sole dashboard (first tab); delete the
  legacy 13-KPI sheet per request (recoverable from Git history)
- Move the 'product points' input into the dashboard (local F31) so the fuel-
  availability formula no longer depends on the removed sheet (no #REF!)
- Update management-reference mapping column to the new K1..K9 numbering
- Point verify_formulas.py at the single dashboard (17 cells: 12 KPIs + 5 axis
  roll-ups), all passing via pycel
- Refresh README to describe the consolidated 9-KPI workbook

https://claude.ai/code/session_01KvBXTcUzJa33dDsqskcTMw
</commit_message>
<xml_diff>
--- a/workbook/khadija-supply-chain-kpis-2026.xlsx
+++ b/workbook/khadija-supply-chain-kpis-2026.xlsx
@@ -7,14 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="📊 ملخص آلي + KPIs" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="📊 لوحة مُكثّفة (٩ مؤشرات)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="📋 مؤشرات الإدارة" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="🛢️ انقطاعات الوقود" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="💧 الردود والفاقد" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="📦 المخزون" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="🛒 الطلبات والمشتريات" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="🚚 النقل والرحلات" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="📊 مؤشرات الأداء (٩)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="📋 مؤشرات الإدارة" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="🛢️ انقطاعات الوقود" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="💧 الردود والفاقد" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="📦 المخزون" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="🛒 الطلبات والمشتريات" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="🚚 النقل والرحلات" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -388,7 +387,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="117">
+  <cellXfs count="119">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -736,6 +735,12 @@
     <xf numFmtId="165" fontId="24" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1062,1877 +1067,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <dimension ref="A1:R39"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
-  <cols>
-    <col width="4" customWidth="1" style="39" min="1" max="1"/>
-    <col width="36" customWidth="1" style="39" min="2" max="2"/>
-    <col width="10" customWidth="1" style="39" min="3" max="3"/>
-    <col width="12" customWidth="1" style="39" min="4" max="4"/>
-    <col width="8" customWidth="1" style="39" min="5" max="5"/>
-    <col width="14" customWidth="1" style="39" min="6" max="6"/>
-    <col width="9" customWidth="1" style="39" min="7" max="18"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="31.5" customHeight="1" s="40">
-      <c r="A1" s="41" t="inlineStr">
-        <is>
-          <t>📊 مؤشرات أداء سلاسل الإمداد 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="27.75" customHeight="1" s="40">
-      <c r="A2" s="42" t="inlineStr">
-        <is>
-          <t>🎯 13 مؤشر عبر 5 محاور · خطة (يدوي) vs فعلي (آلي) · الانحراف يقارن المتوسطين</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="24" customHeight="1" s="40">
-      <c r="A3" s="43" t="inlineStr">
-        <is>
-          <t>📌 المؤشر</t>
-        </is>
-      </c>
-      <c r="G3" s="44" t="inlineStr">
-        <is>
-          <t>📅 الأشهر — خطة (يدوي) vs فعلي (آلي)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1" s="40">
-      <c r="A4" s="45" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B4" s="45" t="inlineStr">
-        <is>
-          <t>المؤشر</t>
-        </is>
-      </c>
-      <c r="C4" s="45" t="inlineStr">
-        <is>
-          <t>الوحدة</t>
-        </is>
-      </c>
-      <c r="D4" s="45" t="inlineStr">
-        <is>
-          <t>الهدف</t>
-        </is>
-      </c>
-      <c r="E4" s="45" t="inlineStr">
-        <is>
-          <t>النوع</t>
-        </is>
-      </c>
-      <c r="F4" s="45" t="inlineStr">
-        <is>
-          <t>الانحراف</t>
-        </is>
-      </c>
-      <c r="G4" s="45" t="inlineStr">
-        <is>
-          <t>يناير</t>
-        </is>
-      </c>
-      <c r="H4" s="45" t="inlineStr">
-        <is>
-          <t>فبراير</t>
-        </is>
-      </c>
-      <c r="I4" s="45" t="inlineStr">
-        <is>
-          <t>مارس</t>
-        </is>
-      </c>
-      <c r="J4" s="45" t="inlineStr">
-        <is>
-          <t>أبريل</t>
-        </is>
-      </c>
-      <c r="K4" s="45" t="inlineStr">
-        <is>
-          <t>مايو</t>
-        </is>
-      </c>
-      <c r="L4" s="45" t="inlineStr">
-        <is>
-          <t>يونيو</t>
-        </is>
-      </c>
-      <c r="M4" s="45" t="inlineStr">
-        <is>
-          <t>يوليو</t>
-        </is>
-      </c>
-      <c r="N4" s="45" t="inlineStr">
-        <is>
-          <t>أغسطس</t>
-        </is>
-      </c>
-      <c r="O4" s="45" t="inlineStr">
-        <is>
-          <t>سبتمبر</t>
-        </is>
-      </c>
-      <c r="P4" s="45" t="inlineStr">
-        <is>
-          <t>أكتوبر</t>
-        </is>
-      </c>
-      <c r="Q4" s="45" t="inlineStr">
-        <is>
-          <t>نوفمبر</t>
-        </is>
-      </c>
-      <c r="R4" s="45" t="inlineStr">
-        <is>
-          <t>ديسمبر</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="25.5" customHeight="1" s="40">
-      <c r="A5" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ◀ 👥 خدمة العميل</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="21.75" customHeight="1" s="40">
-      <c r="A6" s="47" t="n">
-        <v>1</v>
-      </c>
-      <c r="B6" s="48" t="inlineStr">
-        <is>
-          <t>توفر الوقود (1 - نسبة الانقطاع)</t>
-        </is>
-      </c>
-      <c r="C6" s="49" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D6" s="109" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="E6" s="51" t="inlineStr">
-        <is>
-          <t>خطة</t>
-        </is>
-      </c>
-      <c r="F6" s="52" t="n"/>
-      <c r="G6" s="53" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="H6" s="53" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="I6" s="53" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="J6" s="53" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="K6" s="53" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="L6" s="53" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="M6" s="53" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="N6" s="53" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="O6" s="53" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="P6" s="53" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="Q6" s="53" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="R6" s="53" t="n">
-        <v>0.995</v>
-      </c>
-    </row>
-    <row r="7" ht="21.75" customHeight="1" s="40">
-      <c r="A7" s="54" t="n"/>
-      <c r="B7" s="54" t="n"/>
-      <c r="C7" s="54" t="n"/>
-      <c r="D7" s="54" t="n"/>
-      <c r="E7" s="55" t="inlineStr">
-        <is>
-          <t>فعلي</t>
-        </is>
-      </c>
-      <c r="F7" s="56">
-        <f>IFERROR(IF(AVERAGE(G6:R6)=0,"",IF(IFERROR(AVERAGEIF(G7:R7,"&gt;0",G7:R7),0)&gt;=AVERAGE(G6:R6),"✅ ",IF(IFERROR(AVERAGEIF(G7:R7,"&gt;0",G7:R7),0)&gt;=AVERAGE(G6:R6)*0.85,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G7:R7,"&gt;0",G7:R7),0)-AVERAGE(G6:R6))/AVERAGE(G6:R6),"+0.0%;-0.0%")),"")</f>
-        <v/>
-      </c>
-      <c r="G7" s="57">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,1,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,1+1,1))/($F$38*DAY(DATE(2026,1+1,1)-1))),1)</f>
-        <v/>
-      </c>
-      <c r="H7" s="57">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,2,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,2+1,1))/($F$38*DAY(DATE(2026,2+1,1)-1))),1)</f>
-        <v/>
-      </c>
-      <c r="I7" s="57">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,3,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,3+1,1))/($F$38*DAY(DATE(2026,3+1,1)-1))),1)</f>
-        <v/>
-      </c>
-      <c r="J7" s="57">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,4,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,4+1,1))/($F$38*DAY(DATE(2026,4+1,1)-1))),1)</f>
-        <v/>
-      </c>
-      <c r="K7" s="57">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,5,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,5+1,1))/($F$38*DAY(DATE(2026,5+1,1)-1))),1)</f>
-        <v/>
-      </c>
-      <c r="L7" s="57">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,6,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,6+1,1))/($F$38*DAY(DATE(2026,6+1,1)-1))),1)</f>
-        <v/>
-      </c>
-      <c r="M7" s="57">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,7,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,7+1,1))/($F$38*DAY(DATE(2026,7+1,1)-1))),1)</f>
-        <v/>
-      </c>
-      <c r="N7" s="57">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,8,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,8+1,1))/($F$38*DAY(DATE(2026,8+1,1)-1))),1)</f>
-        <v/>
-      </c>
-      <c r="O7" s="57">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,9,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,9+1,1))/($F$38*DAY(DATE(2026,9+1,1)-1))),1)</f>
-        <v/>
-      </c>
-      <c r="P7" s="57">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,10,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,10+1,1))/($F$38*DAY(DATE(2026,10+1,1)-1))),1)</f>
-        <v/>
-      </c>
-      <c r="Q7" s="57">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,11,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,11+1,1))/($F$38*DAY(DATE(2026,11+1,1)-1))),1)</f>
-        <v/>
-      </c>
-      <c r="R7" s="57">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,12,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,12+1,1))/($F$38*DAY(DATE(2026,12+1,1)-1))),1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8" ht="21.75" customHeight="1" s="40">
-      <c r="A8" s="47" t="n">
-        <v>2</v>
-      </c>
-      <c r="B8" s="48" t="inlineStr">
-        <is>
-          <t>عدد الانقطاعات الشهرية</t>
-        </is>
-      </c>
-      <c r="C8" s="49" t="inlineStr">
-        <is>
-          <t>انقطاع</t>
-        </is>
-      </c>
-      <c r="D8" s="110" t="n">
-        <v>5</v>
-      </c>
-      <c r="E8" s="51" t="inlineStr">
-        <is>
-          <t>خطة</t>
-        </is>
-      </c>
-      <c r="F8" s="52" t="n"/>
-      <c r="G8" s="58" t="n">
-        <v>5</v>
-      </c>
-      <c r="H8" s="58" t="n">
-        <v>5</v>
-      </c>
-      <c r="I8" s="58" t="n">
-        <v>5</v>
-      </c>
-      <c r="J8" s="58" t="n">
-        <v>5</v>
-      </c>
-      <c r="K8" s="58" t="n">
-        <v>5</v>
-      </c>
-      <c r="L8" s="58" t="n">
-        <v>5</v>
-      </c>
-      <c r="M8" s="58" t="n">
-        <v>5</v>
-      </c>
-      <c r="N8" s="58" t="n">
-        <v>5</v>
-      </c>
-      <c r="O8" s="58" t="n">
-        <v>5</v>
-      </c>
-      <c r="P8" s="58" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q8" s="58" t="n">
-        <v>5</v>
-      </c>
-      <c r="R8" s="58" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" ht="21.75" customHeight="1" s="40">
-      <c r="A9" s="54" t="n"/>
-      <c r="B9" s="54" t="n"/>
-      <c r="C9" s="54" t="n"/>
-      <c r="D9" s="54" t="n"/>
-      <c r="E9" s="55" t="inlineStr">
-        <is>
-          <t>فعلي</t>
-        </is>
-      </c>
-      <c r="F9" s="56">
-        <f>IFERROR(IF(AVERAGE(G8:R8)=0,"",IF(IFERROR(AVERAGEIF(G9:R9,"&gt;0",G9:R9),0)&lt;=AVERAGE(G8:R8),"✅ ",IF(IFERROR(AVERAGEIF(G9:R9,"&gt;0",G9:R9),0)&lt;=AVERAGE(G8:R8)*1.3,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G9:R9,"&gt;0",G9:R9),0)-AVERAGE(G8:R8))/AVERAGE(G8:R8),"+0.0%;-0.0%")),"")</f>
-        <v/>
-      </c>
-      <c r="G9" s="59">
-        <f>COUNTIFS('🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,1,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,1+1,1))</f>
-        <v/>
-      </c>
-      <c r="H9" s="59">
-        <f>COUNTIFS('🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,2,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,2+1,1))</f>
-        <v/>
-      </c>
-      <c r="I9" s="59">
-        <f>COUNTIFS('🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,3,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,3+1,1))</f>
-        <v/>
-      </c>
-      <c r="J9" s="59">
-        <f>COUNTIFS('🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,4,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,4+1,1))</f>
-        <v/>
-      </c>
-      <c r="K9" s="59">
-        <f>COUNTIFS('🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,5,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,5+1,1))</f>
-        <v/>
-      </c>
-      <c r="L9" s="59">
-        <f>COUNTIFS('🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,6,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,6+1,1))</f>
-        <v/>
-      </c>
-      <c r="M9" s="59">
-        <f>COUNTIFS('🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,7,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,7+1,1))</f>
-        <v/>
-      </c>
-      <c r="N9" s="59">
-        <f>COUNTIFS('🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,8,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,8+1,1))</f>
-        <v/>
-      </c>
-      <c r="O9" s="59">
-        <f>COUNTIFS('🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,9,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,9+1,1))</f>
-        <v/>
-      </c>
-      <c r="P9" s="59">
-        <f>COUNTIFS('🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,10,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,10+1,1))</f>
-        <v/>
-      </c>
-      <c r="Q9" s="59">
-        <f>COUNTIFS('🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,11,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,11+1,1))</f>
-        <v/>
-      </c>
-      <c r="R9" s="59">
-        <f>COUNTIFS('🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,12,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,12+1,1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="21.75" customHeight="1" s="40">
-      <c r="A10" s="47" t="n">
-        <v>3</v>
-      </c>
-      <c r="B10" s="48" t="inlineStr">
-        <is>
-          <t>توفر المواد المخزنية (تسليم ≤ 3 أيام)</t>
-        </is>
-      </c>
-      <c r="C10" s="49" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D10" s="111" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" s="51" t="inlineStr">
-        <is>
-          <t>خطة</t>
-        </is>
-      </c>
-      <c r="F10" s="52" t="n"/>
-      <c r="G10" s="60" t="n">
-        <v>1</v>
-      </c>
-      <c r="H10" s="60" t="n">
-        <v>1</v>
-      </c>
-      <c r="I10" s="60" t="n">
-        <v>1</v>
-      </c>
-      <c r="J10" s="60" t="n">
-        <v>1</v>
-      </c>
-      <c r="K10" s="60" t="n">
-        <v>1</v>
-      </c>
-      <c r="L10" s="60" t="n">
-        <v>1</v>
-      </c>
-      <c r="M10" s="60" t="n">
-        <v>1</v>
-      </c>
-      <c r="N10" s="60" t="n">
-        <v>1</v>
-      </c>
-      <c r="O10" s="60" t="n">
-        <v>1</v>
-      </c>
-      <c r="P10" s="60" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q10" s="60" t="n">
-        <v>1</v>
-      </c>
-      <c r="R10" s="60" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" ht="21.75" customHeight="1" s="40">
-      <c r="A11" s="54" t="n"/>
-      <c r="B11" s="54" t="n"/>
-      <c r="C11" s="54" t="n"/>
-      <c r="D11" s="54" t="n"/>
-      <c r="E11" s="55" t="inlineStr">
-        <is>
-          <t>فعلي</t>
-        </is>
-      </c>
-      <c r="F11" s="56">
-        <f>IFERROR(IF(AVERAGE(G10:R10)=0,"",IF(IFERROR(AVERAGEIF(G11:R11,"&gt;0",G11:R11),0)&gt;=AVERAGE(G10:R10),"✅ ",IF(IFERROR(AVERAGEIF(G11:R11,"&gt;0",G11:R11),0)&gt;=AVERAGE(G10:R10)*0.85,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G11:R11,"&gt;0",G11:R11),0)-AVERAGE(G10:R10))/AVERAGE(G10:R10),"+0.0%;-0.0%")),"")</f>
-        <v/>
-      </c>
-      <c r="G11" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,1,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,1+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,1,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,1+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
-        <v/>
-      </c>
-      <c r="H11" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,2,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,2+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,2,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,2+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
-        <v/>
-      </c>
-      <c r="I11" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,3,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,3+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,3,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,3+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
-        <v/>
-      </c>
-      <c r="J11" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,4,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,4+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,4,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,4+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
-        <v/>
-      </c>
-      <c r="K11" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,5,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,5+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,5,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,5+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
-        <v/>
-      </c>
-      <c r="L11" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,6,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,6+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,6,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,6+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
-        <v/>
-      </c>
-      <c r="M11" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,7,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,7+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,7,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,7+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
-        <v/>
-      </c>
-      <c r="N11" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,8,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,8+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,8,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,8+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
-        <v/>
-      </c>
-      <c r="O11" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,9,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,9+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,9,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,9+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
-        <v/>
-      </c>
-      <c r="P11" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,10,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,10+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,10,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,10+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
-        <v/>
-      </c>
-      <c r="Q11" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,11,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,11+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,11,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,11+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
-        <v/>
-      </c>
-      <c r="R11" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,12,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,12+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,12,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,12+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12" ht="21.75" customHeight="1" s="40">
-      <c r="A12" s="47" t="n">
-        <v>4</v>
-      </c>
-      <c r="B12" s="48" t="inlineStr">
-        <is>
-          <t>إصدار أوامر الشراء (≤ 5 أيام عمل)</t>
-        </is>
-      </c>
-      <c r="C12" s="49" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D12" s="111" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="E12" s="51" t="inlineStr">
-        <is>
-          <t>خطة</t>
-        </is>
-      </c>
-      <c r="F12" s="52" t="n"/>
-      <c r="G12" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="H12" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="I12" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="J12" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="K12" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="L12" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="M12" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="N12" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="O12" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="P12" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="Q12" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="R12" s="60" t="n">
-        <v>0.95</v>
-      </c>
-    </row>
-    <row r="13" ht="21.75" customHeight="1" s="40">
-      <c r="A13" s="54" t="n"/>
-      <c r="B13" s="54" t="n"/>
-      <c r="C13" s="54" t="n"/>
-      <c r="D13" s="54" t="n"/>
-      <c r="E13" s="55" t="inlineStr">
-        <is>
-          <t>فعلي</t>
-        </is>
-      </c>
-      <c r="F13" s="56">
-        <f>IFERROR(IF(AVERAGE(G12:R12)=0,"",IF(IFERROR(AVERAGEIF(G13:R13,"&gt;0",G13:R13),0)&gt;=AVERAGE(G12:R12),"✅ ",IF(IFERROR(AVERAGEIF(G13:R13,"&gt;0",G13:R13),0)&gt;=AVERAGE(G12:R12)*0.85,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G13:R13,"&gt;0",G13:R13),0)-AVERAGE(G12:R12))/AVERAGE(G12:R12),"+0.0%;-0.0%")),"")</f>
-        <v/>
-      </c>
-      <c r="G13" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,1,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,1+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,1,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,1+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
-        <v/>
-      </c>
-      <c r="H13" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,2,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,2+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,2,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,2+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
-        <v/>
-      </c>
-      <c r="I13" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,3,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,3+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,3,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,3+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
-        <v/>
-      </c>
-      <c r="J13" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,4,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,4+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,4,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,4+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
-        <v/>
-      </c>
-      <c r="K13" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,5,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,5+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,5,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,5+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
-        <v/>
-      </c>
-      <c r="L13" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,6,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,6+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,6,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,6+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
-        <v/>
-      </c>
-      <c r="M13" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,7,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,7+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,7,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,7+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
-        <v/>
-      </c>
-      <c r="N13" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,8,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,8+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,8,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,8+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
-        <v/>
-      </c>
-      <c r="O13" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,9,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,9+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,9,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,9+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
-        <v/>
-      </c>
-      <c r="P13" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,10,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,10+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,10,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,10+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
-        <v/>
-      </c>
-      <c r="Q13" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,11,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,11+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,11,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,11+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
-        <v/>
-      </c>
-      <c r="R13" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,12,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,12+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,12,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,12+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" ht="21.75" customHeight="1" s="40">
-      <c r="A14" s="47" t="n">
-        <v>5</v>
-      </c>
-      <c r="B14" s="48" t="inlineStr">
-        <is>
-          <t>نسبة استيفاء طلبات المحطات (Fill Rate)</t>
-        </is>
-      </c>
-      <c r="C14" s="49" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D14" s="111" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="E14" s="51" t="inlineStr">
-        <is>
-          <t>خطة</t>
-        </is>
-      </c>
-      <c r="F14" s="52" t="n"/>
-      <c r="G14" s="60" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="H14" s="60" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="I14" s="60" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="J14" s="60" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="K14" s="60" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="L14" s="60" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="M14" s="60" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="N14" s="60" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="O14" s="60" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="P14" s="60" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="Q14" s="60" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="R14" s="60" t="n">
-        <v>0.98</v>
-      </c>
-    </row>
-    <row r="15" ht="21.75" customHeight="1" s="40">
-      <c r="A15" s="54" t="n"/>
-      <c r="B15" s="54" t="n"/>
-      <c r="C15" s="54" t="n"/>
-      <c r="D15" s="54" t="n"/>
-      <c r="E15" s="55" t="inlineStr">
-        <is>
-          <t>فعلي</t>
-        </is>
-      </c>
-      <c r="F15" s="56">
-        <f>IFERROR(IF(AVERAGE(G14:R14)=0,"",IF(IFERROR(AVERAGEIF(G15:R15,"&gt;0",G15:R15),0)&gt;=AVERAGE(G14:R14),"✅ ",IF(IFERROR(AVERAGEIF(G15:R15,"&gt;0",G15:R15),0)&gt;=AVERAGE(G14:R14)*0.85,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G15:R15,"&gt;0",G15:R15),0)-AVERAGE(G14:R14))/AVERAGE(G14:R14),"+0.0%;-0.0%")),"")</f>
-        <v/>
-      </c>
-      <c r="G15" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,1,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,1+1,1),'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,1,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,1+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="H15" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,2,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,2+1,1),'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,2,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,2+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="I15" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,3,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,3+1,1),'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,3,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,3+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="J15" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,4,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,4+1,1),'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,4,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,4+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="K15" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,5,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,5+1,1),'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,5,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,5+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="L15" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,6,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,6+1,1),'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,6,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,6+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="M15" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,7,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,7+1,1),'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,7,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,7+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="N15" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,8,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,8+1,1),'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,8,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,8+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="O15" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,9,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,9+1,1),'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,9,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,9+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="P15" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,10,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,10+1,1),'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,10,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,10+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="Q15" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,11,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,11+1,1),'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,11,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,11+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="R15" s="61">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,12,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,12+1,1),'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,12,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,12+1,1))),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" ht="25.5" customHeight="1" s="40">
-      <c r="A16" s="62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ◀ 💰 التكاليف</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="21.75" customHeight="1" s="40">
-      <c r="A17" s="47" t="n">
-        <v>6</v>
-      </c>
-      <c r="B17" s="48" t="inlineStr">
-        <is>
-          <t>فواقد الوقود لكل 33K لتر</t>
-        </is>
-      </c>
-      <c r="C17" s="49" t="inlineStr">
-        <is>
-          <t>لتر</t>
-        </is>
-      </c>
-      <c r="D17" s="112" t="n">
-        <v>100</v>
-      </c>
-      <c r="E17" s="51" t="inlineStr">
-        <is>
-          <t>خطة</t>
-        </is>
-      </c>
-      <c r="F17" s="52" t="n"/>
-      <c r="G17" s="63" t="n">
-        <v>100</v>
-      </c>
-      <c r="H17" s="63" t="n">
-        <v>100</v>
-      </c>
-      <c r="I17" s="63" t="n">
-        <v>100</v>
-      </c>
-      <c r="J17" s="63" t="n">
-        <v>100</v>
-      </c>
-      <c r="K17" s="63" t="n">
-        <v>100</v>
-      </c>
-      <c r="L17" s="63" t="n">
-        <v>100</v>
-      </c>
-      <c r="M17" s="63" t="n">
-        <v>100</v>
-      </c>
-      <c r="N17" s="63" t="n">
-        <v>100</v>
-      </c>
-      <c r="O17" s="63" t="n">
-        <v>100</v>
-      </c>
-      <c r="P17" s="63" t="n">
-        <v>100</v>
-      </c>
-      <c r="Q17" s="63" t="n">
-        <v>100</v>
-      </c>
-      <c r="R17" s="63" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="18" ht="21.75" customHeight="1" s="40">
-      <c r="A18" s="54" t="n"/>
-      <c r="B18" s="54" t="n"/>
-      <c r="C18" s="54" t="n"/>
-      <c r="D18" s="54" t="n"/>
-      <c r="E18" s="55" t="inlineStr">
-        <is>
-          <t>فعلي</t>
-        </is>
-      </c>
-      <c r="F18" s="56">
-        <f>IFERROR(IF(AVERAGE(G17:R17)=0,"",IF(IFERROR(AVERAGEIF(G18:R18,"&gt;0",G18:R18),0)&lt;=AVERAGE(G17:R17),"✅ ",IF(IFERROR(AVERAGEIF(G18:R18,"&gt;0",G18:R18),0)&lt;=AVERAGE(G17:R17)*1.3,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G18:R18,"&gt;0",G18:R18),0)-AVERAGE(G17:R17))/AVERAGE(G17:R17),"+0.0%;-0.0%")),"")</f>
-        <v/>
-      </c>
-      <c r="G18" s="64">
-        <f>IFERROR(SUMIFS('💧 الردود والفاقد'!G5:G304,'💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,1,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,1+1,1))/COUNTIFS('💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,1,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,1+1,1)),0)</f>
-        <v/>
-      </c>
-      <c r="H18" s="64">
-        <f>IFERROR(SUMIFS('💧 الردود والفاقد'!G5:G304,'💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,2,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,2+1,1))/COUNTIFS('💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,2,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,2+1,1)),0)</f>
-        <v/>
-      </c>
-      <c r="I18" s="64">
-        <f>IFERROR(SUMIFS('💧 الردود والفاقد'!G5:G304,'💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,3,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,3+1,1))/COUNTIFS('💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,3,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,3+1,1)),0)</f>
-        <v/>
-      </c>
-      <c r="J18" s="64">
-        <f>IFERROR(SUMIFS('💧 الردود والفاقد'!G5:G304,'💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,4,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,4+1,1))/COUNTIFS('💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,4,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,4+1,1)),0)</f>
-        <v/>
-      </c>
-      <c r="K18" s="64">
-        <f>IFERROR(SUMIFS('💧 الردود والفاقد'!G5:G304,'💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,5,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,5+1,1))/COUNTIFS('💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,5,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,5+1,1)),0)</f>
-        <v/>
-      </c>
-      <c r="L18" s="64">
-        <f>IFERROR(SUMIFS('💧 الردود والفاقد'!G5:G304,'💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,6,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,6+1,1))/COUNTIFS('💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,6,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,6+1,1)),0)</f>
-        <v/>
-      </c>
-      <c r="M18" s="64">
-        <f>IFERROR(SUMIFS('💧 الردود والفاقد'!G5:G304,'💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,7,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,7+1,1))/COUNTIFS('💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,7,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,7+1,1)),0)</f>
-        <v/>
-      </c>
-      <c r="N18" s="64">
-        <f>IFERROR(SUMIFS('💧 الردود والفاقد'!G5:G304,'💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,8,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,8+1,1))/COUNTIFS('💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,8,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,8+1,1)),0)</f>
-        <v/>
-      </c>
-      <c r="O18" s="64">
-        <f>IFERROR(SUMIFS('💧 الردود والفاقد'!G5:G304,'💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,9,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,9+1,1))/COUNTIFS('💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,9,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,9+1,1)),0)</f>
-        <v/>
-      </c>
-      <c r="P18" s="64">
-        <f>IFERROR(SUMIFS('💧 الردود والفاقد'!G5:G304,'💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,10,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,10+1,1))/COUNTIFS('💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,10,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,10+1,1)),0)</f>
-        <v/>
-      </c>
-      <c r="Q18" s="64">
-        <f>IFERROR(SUMIFS('💧 الردود والفاقد'!G5:G304,'💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,11,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,11+1,1))/COUNTIFS('💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,11,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,11+1,1)),0)</f>
-        <v/>
-      </c>
-      <c r="R18" s="64">
-        <f>IFERROR(SUMIFS('💧 الردود والفاقد'!G5:G304,'💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,12,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,12+1,1))/COUNTIFS('💧 الردود والفاقد'!B5:B304,"&gt;="&amp;DATE(2026,12,1),'💧 الردود والفاقد'!B5:B304,"&lt;"&amp;DATE(2026,12+1,1)),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" ht="21.75" customHeight="1" s="40">
-      <c r="A19" s="47" t="n">
-        <v>7</v>
-      </c>
-      <c r="B19" s="48" t="inlineStr">
-        <is>
-          <t>نسبة المواد التالفة (يدوي شهرياً)</t>
-        </is>
-      </c>
-      <c r="C19" s="49" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D19" s="111" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="E19" s="51" t="inlineStr">
-        <is>
-          <t>خطة</t>
-        </is>
-      </c>
-      <c r="F19" s="52" t="n"/>
-      <c r="G19" s="60" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="H19" s="60" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="I19" s="60" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="J19" s="60" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="K19" s="60" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="L19" s="60" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="M19" s="60" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="N19" s="60" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="O19" s="60" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="P19" s="60" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="Q19" s="60" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="R19" s="60" t="n">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="20" ht="21.75" customHeight="1" s="40">
-      <c r="A20" s="54" t="n"/>
-      <c r="B20" s="54" t="n"/>
-      <c r="C20" s="54" t="n"/>
-      <c r="D20" s="54" t="n"/>
-      <c r="E20" s="55" t="inlineStr">
-        <is>
-          <t>فعلي</t>
-        </is>
-      </c>
-      <c r="F20" s="56">
-        <f>IFERROR(IF(AVERAGE(G19:R19)=0,"",IF(IFERROR(AVERAGEIF(G20:R20,"&gt;0",G20:R20),0)&lt;=AVERAGE(G19:R19),"✅ ",IF(IFERROR(AVERAGEIF(G20:R20,"&gt;0",G20:R20),0)&lt;=AVERAGE(G19:R19)*1.3,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G20:R20,"&gt;0",G20:R20),0)-AVERAGE(G19:R19))/AVERAGE(G19:R19),"+0.0%;-0.0%")),"")</f>
-        <v/>
-      </c>
-      <c r="G20" s="61" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" s="61" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" s="61" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" s="61" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" s="61" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" s="61" t="n">
-        <v>0</v>
-      </c>
-      <c r="M20" s="61" t="n">
-        <v>0</v>
-      </c>
-      <c r="N20" s="61" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" s="61" t="n">
-        <v>0</v>
-      </c>
-      <c r="P20" s="61" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q20" s="61" t="n">
-        <v>0</v>
-      </c>
-      <c r="R20" s="61" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" ht="25.5" customHeight="1" s="40">
-      <c r="A21" s="65" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ◀ 🏦 السيولة المالية</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="21.75" customHeight="1" s="40">
-      <c r="A22" s="47" t="n">
-        <v>8</v>
-      </c>
-      <c r="B22" s="48" t="inlineStr">
-        <is>
-          <t>كمية مخزون الوقود (أيام)</t>
-        </is>
-      </c>
-      <c r="C22" s="49" t="inlineStr">
-        <is>
-          <t>يوم</t>
-        </is>
-      </c>
-      <c r="D22" s="112" t="n">
-        <v>3</v>
-      </c>
-      <c r="E22" s="51" t="inlineStr">
-        <is>
-          <t>خطة</t>
-        </is>
-      </c>
-      <c r="F22" s="52" t="n"/>
-      <c r="G22" s="63" t="n">
-        <v>3</v>
-      </c>
-      <c r="H22" s="63" t="n">
-        <v>3</v>
-      </c>
-      <c r="I22" s="63" t="n">
-        <v>3</v>
-      </c>
-      <c r="J22" s="63" t="n">
-        <v>3</v>
-      </c>
-      <c r="K22" s="63" t="n">
-        <v>3</v>
-      </c>
-      <c r="L22" s="63" t="n">
-        <v>3</v>
-      </c>
-      <c r="M22" s="63" t="n">
-        <v>3</v>
-      </c>
-      <c r="N22" s="63" t="n">
-        <v>3</v>
-      </c>
-      <c r="O22" s="63" t="n">
-        <v>3</v>
-      </c>
-      <c r="P22" s="63" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q22" s="63" t="n">
-        <v>3</v>
-      </c>
-      <c r="R22" s="63" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" ht="21.75" customHeight="1" s="40">
-      <c r="A23" s="54" t="n"/>
-      <c r="B23" s="54" t="n"/>
-      <c r="C23" s="54" t="n"/>
-      <c r="D23" s="54" t="n"/>
-      <c r="E23" s="55" t="inlineStr">
-        <is>
-          <t>فعلي</t>
-        </is>
-      </c>
-      <c r="F23" s="56">
-        <f>IFERROR(IF(AVERAGE(G22:R22)=0,"",IF(IFERROR(AVERAGEIF(G23:R23,"&gt;0",G23:R23),0)&lt;=AVERAGE(G22:R22),"✅ ",IF(IFERROR(AVERAGEIF(G23:R23,"&gt;0",G23:R23),0)&lt;=AVERAGE(G22:R22)*1.3,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G23:R23,"&gt;0",G23:R23),0)-AVERAGE(G22:R22))/AVERAGE(G22:R22),"+0.0%;-0.0%")),"")</f>
-        <v/>
-      </c>
-      <c r="G23" s="64">
-        <f>IFERROR(AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,1,'📦 المخزون'!F5:F304,"وقود"),0)</f>
-        <v/>
-      </c>
-      <c r="H23" s="64">
-        <f>IFERROR(AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,2,'📦 المخزون'!F5:F304,"وقود"),0)</f>
-        <v/>
-      </c>
-      <c r="I23" s="64">
-        <f>IFERROR(AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,3,'📦 المخزون'!F5:F304,"وقود"),0)</f>
-        <v/>
-      </c>
-      <c r="J23" s="64">
-        <f>IFERROR(AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,4,'📦 المخزون'!F5:F304,"وقود"),0)</f>
-        <v/>
-      </c>
-      <c r="K23" s="64">
-        <f>IFERROR(AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,5,'📦 المخزون'!F5:F304,"وقود"),0)</f>
-        <v/>
-      </c>
-      <c r="L23" s="64">
-        <f>IFERROR(AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,6,'📦 المخزون'!F5:F304,"وقود"),0)</f>
-        <v/>
-      </c>
-      <c r="M23" s="64">
-        <f>IFERROR(AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,7,'📦 المخزون'!F5:F304,"وقود"),0)</f>
-        <v/>
-      </c>
-      <c r="N23" s="64">
-        <f>IFERROR(AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,8,'📦 المخزون'!F5:F304,"وقود"),0)</f>
-        <v/>
-      </c>
-      <c r="O23" s="64">
-        <f>IFERROR(AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,9,'📦 المخزون'!F5:F304,"وقود"),0)</f>
-        <v/>
-      </c>
-      <c r="P23" s="64">
-        <f>IFERROR(AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,10,'📦 المخزون'!F5:F304,"وقود"),0)</f>
-        <v/>
-      </c>
-      <c r="Q23" s="64">
-        <f>IFERROR(AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,11,'📦 المخزون'!F5:F304,"وقود"),0)</f>
-        <v/>
-      </c>
-      <c r="R23" s="64">
-        <f>IFERROR(AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,12,'📦 المخزون'!F5:F304,"وقود"),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" ht="21.75" customHeight="1" s="40">
-      <c r="A24" s="47" t="n">
-        <v>9</v>
-      </c>
-      <c r="B24" s="48" t="inlineStr">
-        <is>
-          <t>معدل دوران المخزون (مرات/شهر)</t>
-        </is>
-      </c>
-      <c r="C24" s="49" t="inlineStr">
-        <is>
-          <t>مرة</t>
-        </is>
-      </c>
-      <c r="D24" s="112" t="n">
-        <v>10</v>
-      </c>
-      <c r="E24" s="51" t="inlineStr">
-        <is>
-          <t>خطة</t>
-        </is>
-      </c>
-      <c r="F24" s="52" t="n"/>
-      <c r="G24" s="63" t="n">
-        <v>10</v>
-      </c>
-      <c r="H24" s="63" t="n">
-        <v>10</v>
-      </c>
-      <c r="I24" s="63" t="n">
-        <v>10</v>
-      </c>
-      <c r="J24" s="63" t="n">
-        <v>10</v>
-      </c>
-      <c r="K24" s="63" t="n">
-        <v>10</v>
-      </c>
-      <c r="L24" s="63" t="n">
-        <v>10</v>
-      </c>
-      <c r="M24" s="63" t="n">
-        <v>10</v>
-      </c>
-      <c r="N24" s="63" t="n">
-        <v>10</v>
-      </c>
-      <c r="O24" s="63" t="n">
-        <v>10</v>
-      </c>
-      <c r="P24" s="63" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q24" s="63" t="n">
-        <v>10</v>
-      </c>
-      <c r="R24" s="63" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="25" ht="21.75" customHeight="1" s="40">
-      <c r="A25" s="54" t="n"/>
-      <c r="B25" s="54" t="n"/>
-      <c r="C25" s="54" t="n"/>
-      <c r="D25" s="54" t="n"/>
-      <c r="E25" s="55" t="inlineStr">
-        <is>
-          <t>فعلي</t>
-        </is>
-      </c>
-      <c r="F25" s="56">
-        <f>IFERROR(IF(AVERAGE(G24:R24)=0,"",IF(IFERROR(AVERAGEIF(G25:R25,"&gt;0",G25:R25),0)&gt;=AVERAGE(G24:R24),"✅ ",IF(IFERROR(AVERAGEIF(G25:R25,"&gt;0",G25:R25),0)&gt;=AVERAGE(G24:R24)*0.85,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G25:R25,"&gt;0",G25:R25),0)-AVERAGE(G24:R24))/AVERAGE(G24:R24),"+0.0%;-0.0%")),"")</f>
-        <v/>
-      </c>
-      <c r="G25" s="64">
-        <f>IFERROR(30/AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,1,'📦 المخزون'!F5:F304,"وقود"),0)</f>
-        <v/>
-      </c>
-      <c r="H25" s="64">
-        <f>IFERROR(30/AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,2,'📦 المخزون'!F5:F304,"وقود"),0)</f>
-        <v/>
-      </c>
-      <c r="I25" s="64">
-        <f>IFERROR(30/AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,3,'📦 المخزون'!F5:F304,"وقود"),0)</f>
-        <v/>
-      </c>
-      <c r="J25" s="64">
-        <f>IFERROR(30/AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,4,'📦 المخزون'!F5:F304,"وقود"),0)</f>
-        <v/>
-      </c>
-      <c r="K25" s="64">
-        <f>IFERROR(30/AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,5,'📦 المخزون'!F5:F304,"وقود"),0)</f>
-        <v/>
-      </c>
-      <c r="L25" s="64">
-        <f>IFERROR(30/AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,6,'📦 المخزون'!F5:F304,"وقود"),0)</f>
-        <v/>
-      </c>
-      <c r="M25" s="64">
-        <f>IFERROR(30/AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,7,'📦 المخزون'!F5:F304,"وقود"),0)</f>
-        <v/>
-      </c>
-      <c r="N25" s="64">
-        <f>IFERROR(30/AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,8,'📦 المخزون'!F5:F304,"وقود"),0)</f>
-        <v/>
-      </c>
-      <c r="O25" s="64">
-        <f>IFERROR(30/AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,9,'📦 المخزون'!F5:F304,"وقود"),0)</f>
-        <v/>
-      </c>
-      <c r="P25" s="64">
-        <f>IFERROR(30/AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,10,'📦 المخزون'!F5:F304,"وقود"),0)</f>
-        <v/>
-      </c>
-      <c r="Q25" s="64">
-        <f>IFERROR(30/AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,11,'📦 المخزون'!F5:F304,"وقود"),0)</f>
-        <v/>
-      </c>
-      <c r="R25" s="64">
-        <f>IFERROR(30/AVERAGEIFS('📦 المخزون'!I5:I304,'📦 المخزون'!C5:C304,12,'📦 المخزون'!F5:F304,"وقود"),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26" ht="25.5" customHeight="1" s="40">
-      <c r="A26" s="66" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ◀ 🛡️ السلامة والامتثال</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="21.75" customHeight="1" s="40">
-      <c r="A27" s="47" t="n">
-        <v>10</v>
-      </c>
-      <c r="B27" s="48" t="inlineStr">
-        <is>
-          <t>عدد حوادث النقل الشهرية</t>
-        </is>
-      </c>
-      <c r="C27" s="49" t="inlineStr">
-        <is>
-          <t>حادث</t>
-        </is>
-      </c>
-      <c r="D27" s="110" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" s="51" t="inlineStr">
-        <is>
-          <t>خطة</t>
-        </is>
-      </c>
-      <c r="F27" s="52" t="n"/>
-      <c r="G27" s="58" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" s="58" t="n">
-        <v>0</v>
-      </c>
-      <c r="I27" s="58" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" s="58" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" s="58" t="n">
-        <v>0</v>
-      </c>
-      <c r="L27" s="58" t="n">
-        <v>0</v>
-      </c>
-      <c r="M27" s="58" t="n">
-        <v>0</v>
-      </c>
-      <c r="N27" s="58" t="n">
-        <v>0</v>
-      </c>
-      <c r="O27" s="58" t="n">
-        <v>0</v>
-      </c>
-      <c r="P27" s="58" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q27" s="58" t="n">
-        <v>0</v>
-      </c>
-      <c r="R27" s="58" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" ht="21.75" customHeight="1" s="40">
-      <c r="A28" s="54" t="n"/>
-      <c r="B28" s="54" t="n"/>
-      <c r="C28" s="54" t="n"/>
-      <c r="D28" s="54" t="n"/>
-      <c r="E28" s="55" t="inlineStr">
-        <is>
-          <t>فعلي</t>
-        </is>
-      </c>
-      <c r="F28" s="56">
-        <f>IFERROR(IF(AVERAGE(G27:R27)=0,"",IF(IFERROR(AVERAGEIF(G28:R28,"&gt;0",G28:R28),0)&lt;=AVERAGE(G27:R27),"✅ ",IF(IFERROR(AVERAGEIF(G28:R28,"&gt;0",G28:R28),0)&lt;=AVERAGE(G27:R27)*1.3,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G28:R28,"&gt;0",G28:R28),0)-AVERAGE(G27:R27))/AVERAGE(G27:R27),"+0.0%;-0.0%")),"")</f>
-        <v/>
-      </c>
-      <c r="G28" s="59">
-        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,1,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,1+1,1),'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;لا يوجد",'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="H28" s="59">
-        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,2,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,2+1,1),'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;لا يوجد",'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="I28" s="59">
-        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,3,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,3+1,1),'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;لا يوجد",'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="J28" s="59">
-        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,4,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,4+1,1),'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;لا يوجد",'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="K28" s="59">
-        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,5,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,5+1,1),'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;لا يوجد",'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="L28" s="59">
-        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,6,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,6+1,1),'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;لا يوجد",'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="M28" s="59">
-        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,7,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,7+1,1),'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;لا يوجد",'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="N28" s="59">
-        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,8,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,8+1,1),'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;لا يوجد",'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="O28" s="59">
-        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,9,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,9+1,1),'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;لا يوجد",'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="P28" s="59">
-        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,10,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,10+1,1),'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;لا يوجد",'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="Q28" s="59">
-        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,11,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,11+1,1),'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;لا يوجد",'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="R28" s="59">
-        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,12,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,12+1,1),'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;لا يوجد",'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" ht="21.75" customHeight="1" s="40">
-      <c r="A29" s="47" t="n">
-        <v>11</v>
-      </c>
-      <c r="B29" s="48" t="inlineStr">
-        <is>
-          <t>معدل امتثال السائقين (بدون مخالفات)</t>
-        </is>
-      </c>
-      <c r="C29" s="49" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D29" s="111" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="E29" s="51" t="inlineStr">
-        <is>
-          <t>خطة</t>
-        </is>
-      </c>
-      <c r="F29" s="52" t="n"/>
-      <c r="G29" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="H29" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="I29" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="J29" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="K29" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="L29" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="M29" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="N29" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="O29" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="P29" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="Q29" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="R29" s="60" t="n">
-        <v>0.95</v>
-      </c>
-    </row>
-    <row r="30" ht="21.75" customHeight="1" s="40">
-      <c r="A30" s="54" t="n"/>
-      <c r="B30" s="54" t="n"/>
-      <c r="C30" s="54" t="n"/>
-      <c r="D30" s="54" t="n"/>
-      <c r="E30" s="55" t="inlineStr">
-        <is>
-          <t>فعلي</t>
-        </is>
-      </c>
-      <c r="F30" s="56">
-        <f>IFERROR(IF(AVERAGE(G29:R29)=0,"",IF(IFERROR(AVERAGEIF(G30:R30,"&gt;0",G30:R30),0)&gt;=AVERAGE(G29:R29),"✅ ",IF(IFERROR(AVERAGEIF(G30:R30,"&gt;0",G30:R30),0)&gt;=AVERAGE(G29:R29)*0.85,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G30:R30,"&gt;0",G30:R30),0)-AVERAGE(G29:R29))/AVERAGE(G29:R29),"+0.0%;-0.0%")),"")</f>
-        <v/>
-      </c>
-      <c r="G30" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,1,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,1+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,1,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,1+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="H30" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,2,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,2+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,2,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,2+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="I30" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,3,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,3+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,3,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,3+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="J30" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,4,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,4+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,4,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,4+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="K30" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,5,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,5+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,5,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,5+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="L30" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,6,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,6+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,6,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,6+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="M30" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,7,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,7+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,7,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,7+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="N30" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,8,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,8+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,8,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,8+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="O30" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,9,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,9+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,9,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,9+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="P30" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,10,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,10+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,10,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,10+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="Q30" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,11,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,11+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,11,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,11+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="R30" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,12,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,12+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,12,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,12+1,1))),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" ht="25.5" customHeight="1" s="40">
-      <c r="A31" s="67" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ◀ ⚙️ الكفاءة التشغيلية</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="21.75" customHeight="1" s="40">
-      <c r="A32" s="47" t="n">
-        <v>12</v>
-      </c>
-      <c r="B32" s="48" t="inlineStr">
-        <is>
-          <t>التزام جدول النقل (On-time)</t>
-        </is>
-      </c>
-      <c r="C32" s="49" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D32" s="111" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="E32" s="51" t="inlineStr">
-        <is>
-          <t>خطة</t>
-        </is>
-      </c>
-      <c r="F32" s="52" t="n"/>
-      <c r="G32" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="H32" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="I32" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="J32" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="K32" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="L32" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="M32" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="N32" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="O32" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="P32" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="Q32" s="60" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="R32" s="60" t="n">
-        <v>0.95</v>
-      </c>
-    </row>
-    <row r="33" ht="21.75" customHeight="1" s="40">
-      <c r="A33" s="54" t="n"/>
-      <c r="B33" s="54" t="n"/>
-      <c r="C33" s="54" t="n"/>
-      <c r="D33" s="54" t="n"/>
-      <c r="E33" s="55" t="inlineStr">
-        <is>
-          <t>فعلي</t>
-        </is>
-      </c>
-      <c r="F33" s="56">
-        <f>IFERROR(IF(AVERAGE(G32:R32)=0,"",IF(IFERROR(AVERAGEIF(G33:R33,"&gt;0",G33:R33),0)&gt;=AVERAGE(G32:R32),"✅ ",IF(IFERROR(AVERAGEIF(G33:R33,"&gt;0",G33:R33),0)&gt;=AVERAGE(G32:R32)*0.85,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G33:R33,"&gt;0",G33:R33),0)-AVERAGE(G32:R32))/AVERAGE(G32:R32),"+0.0%;-0.0%")),"")</f>
-        <v/>
-      </c>
-      <c r="G33" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,1,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,1+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,1,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,1+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="H33" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,2,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,2+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,2,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,2+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="I33" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,3,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,3+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,3,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,3+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="J33" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,4,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,4+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,4,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,4+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="K33" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,5,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,5+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,5,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,5+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="L33" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,6,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,6+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,6,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,6+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="M33" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,7,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,7+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,7,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,7+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="N33" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,8,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,8+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,8,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,8+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="O33" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,9,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,9+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,9,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,9+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="P33" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,10,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,10+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,10,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,10+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="Q33" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,11,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,11+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,11,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,11+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="R33" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,12,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,12+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,12,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,12+1,1))),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34" ht="21.75" customHeight="1" s="40">
-      <c r="A34" s="47" t="n">
-        <v>13</v>
-      </c>
-      <c r="B34" s="48" t="inlineStr">
-        <is>
-          <t>نسبة استخدام الأسطول المملوك</t>
-        </is>
-      </c>
-      <c r="C34" s="49" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D34" s="111" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E34" s="51" t="inlineStr">
-        <is>
-          <t>خطة</t>
-        </is>
-      </c>
-      <c r="F34" s="52" t="n"/>
-      <c r="G34" s="60" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H34" s="60" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="I34" s="60" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="J34" s="60" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="K34" s="60" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="L34" s="60" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="M34" s="60" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="N34" s="60" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="O34" s="60" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="P34" s="60" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="Q34" s="60" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="R34" s="60" t="n">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="35" ht="21.75" customHeight="1" s="40">
-      <c r="A35" s="54" t="n"/>
-      <c r="B35" s="54" t="n"/>
-      <c r="C35" s="54" t="n"/>
-      <c r="D35" s="54" t="n"/>
-      <c r="E35" s="55" t="inlineStr">
-        <is>
-          <t>فعلي</t>
-        </is>
-      </c>
-      <c r="F35" s="56">
-        <f>IFERROR(IF(AVERAGE(G34:R34)=0,"",IF(IFERROR(AVERAGEIF(G35:R35,"&gt;0",G35:R35),0)&gt;=AVERAGE(G34:R34),"✅ ",IF(IFERROR(AVERAGEIF(G35:R35,"&gt;0",G35:R35),0)&gt;=AVERAGE(G34:R34)*0.85,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G35:R35,"&gt;0",G35:R35),0)-AVERAGE(G34:R34))/AVERAGE(G34:R34),"+0.0%;-0.0%")),"")</f>
-        <v/>
-      </c>
-      <c r="G35" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,1,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,1+1,1),'🚚 النقل والرحلات'!G5:G304,"مملوك درب")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,1,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,1+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="H35" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,2,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,2+1,1),'🚚 النقل والرحلات'!G5:G304,"مملوك درب")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,2,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,2+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="I35" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,3,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,3+1,1),'🚚 النقل والرحلات'!G5:G304,"مملوك درب")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,3,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,3+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="J35" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,4,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,4+1,1),'🚚 النقل والرحلات'!G5:G304,"مملوك درب")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,4,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,4+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="K35" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,5,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,5+1,1),'🚚 النقل والرحلات'!G5:G304,"مملوك درب")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,5,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,5+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="L35" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,6,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,6+1,1),'🚚 النقل والرحلات'!G5:G304,"مملوك درب")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,6,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,6+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="M35" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,7,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,7+1,1),'🚚 النقل والرحلات'!G5:G304,"مملوك درب")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,7,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,7+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="N35" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,8,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,8+1,1),'🚚 النقل والرحلات'!G5:G304,"مملوك درب")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,8,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,8+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="O35" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,9,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,9+1,1),'🚚 النقل والرحلات'!G5:G304,"مملوك درب")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,9,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,9+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="P35" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,10,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,10+1,1),'🚚 النقل والرحلات'!G5:G304,"مملوك درب")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,10,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,10+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="Q35" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,11,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,11+1,1),'🚚 النقل والرحلات'!G5:G304,"مملوك درب")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,11,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,11+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="R35" s="61">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,12,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,12+1,1),'🚚 النقل والرحلات'!G5:G304,"مملوك درب")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,12,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,12+1,1))),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="68" t="inlineStr">
-        <is>
-          <t>⚙️ مُدخلات الحساب اليدوية (حسب طريقة قياس الإدارة)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="69" t="inlineStr">
-        <is>
-          <t>عدد نقاط المنتج (محطات × منتجات) — لحساب «توفر الوقود»</t>
-        </is>
-      </c>
-      <c r="F38" s="70" t="n">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="71" t="inlineStr">
-        <is>
-          <t>ℹ️ الافتراضي 300 = 9000 ÷ 30 (مكافئ للثابت القديم في الأشهر ذات 30 يوماً). غيّره ليعكس عدد (المحطات × المنتجات) الفعلي.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="64">
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="D27:D28"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="A16:R16"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="A37:R37"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="G3:R3"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="A26:R26"/>
-    <mergeCell ref="A21:R21"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="D32:D33"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="A2:R2"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="A5:R5"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="A32:A33"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A22:A23"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="C32:C33"/>
-    <mergeCell ref="A10:A11"/>
-    <mergeCell ref="A31:R31"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="D29:D30"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="A39:R39"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="A34:A35"/>
-    <mergeCell ref="A38:E38"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="C34:C35"/>
-    <mergeCell ref="A1:R1"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="D34:D35"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D22:D23"/>
-  </mergeCells>
-  <conditionalFormatting sqref="F6:F36">
-    <cfRule type="expression" rank="0" priority="2" equalAverage="0" aboveAverage="0" dxfId="0" text="" percent="0" bottom="0">
-      <formula>ISNUMBER(SEARCH("✅",F6))</formula>
-    </cfRule>
-    <cfRule type="expression" rank="0" priority="3" equalAverage="0" aboveAverage="0" dxfId="1" text="" percent="0" bottom="0">
-      <formula>ISNUMBER(SEARCH("🟡",F6))</formula>
-    </cfRule>
-    <cfRule type="expression" rank="0" priority="4" equalAverage="0" aboveAverage="0" dxfId="2" text="" percent="0" bottom="0">
-      <formula>ISNUMBER(SEARCH("🔴",F6))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R29"/>
+  <dimension ref="A1:R31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" style="40" min="1" max="1"/>
@@ -2958,7 +1097,7 @@
     <row r="1" ht="28" customHeight="1" s="40">
       <c r="A1" s="96" t="inlineStr">
         <is>
-          <t>📊 لوحة المؤشرات المُكثّفة — بعد دمج المتكرر (٩ مؤشرات)</t>
+          <t>📊 مؤشرات أداء سلاسل الإمداد ٢٠٢٦ (٩ مؤشرات)</t>
         </is>
       </c>
     </row>
@@ -3156,51 +1295,51 @@
         <v/>
       </c>
       <c r="G7" s="106">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,1,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,1+1,1))/('📊 ملخص آلي + KPIs'!$F$38*DAY(DATE(2026,1+1,1)-1))),1)</f>
+        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,1,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,1+1,1))/($F$31*DAY(DATE(2026,1+1,1)-1))),1)</f>
         <v/>
       </c>
       <c r="H7" s="106">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,2,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,2+1,1))/('📊 ملخص آلي + KPIs'!$F$38*DAY(DATE(2026,2+1,1)-1))),1)</f>
+        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,2,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,2+1,1))/($F$31*DAY(DATE(2026,2+1,1)-1))),1)</f>
         <v/>
       </c>
       <c r="I7" s="106">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,3,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,3+1,1))/('📊 ملخص آلي + KPIs'!$F$38*DAY(DATE(2026,3+1,1)-1))),1)</f>
+        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,3,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,3+1,1))/($F$31*DAY(DATE(2026,3+1,1)-1))),1)</f>
         <v/>
       </c>
       <c r="J7" s="106">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,4,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,4+1,1))/('📊 ملخص آلي + KPIs'!$F$38*DAY(DATE(2026,4+1,1)-1))),1)</f>
+        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,4,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,4+1,1))/($F$31*DAY(DATE(2026,4+1,1)-1))),1)</f>
         <v/>
       </c>
       <c r="K7" s="106">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,5,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,5+1,1))/('📊 ملخص آلي + KPIs'!$F$38*DAY(DATE(2026,5+1,1)-1))),1)</f>
+        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,5,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,5+1,1))/($F$31*DAY(DATE(2026,5+1,1)-1))),1)</f>
         <v/>
       </c>
       <c r="L7" s="106">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,6,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,6+1,1))/('📊 ملخص آلي + KPIs'!$F$38*DAY(DATE(2026,6+1,1)-1))),1)</f>
+        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,6,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,6+1,1))/($F$31*DAY(DATE(2026,6+1,1)-1))),1)</f>
         <v/>
       </c>
       <c r="M7" s="106">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,7,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,7+1,1))/('📊 ملخص آلي + KPIs'!$F$38*DAY(DATE(2026,7+1,1)-1))),1)</f>
+        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,7,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,7+1,1))/($F$31*DAY(DATE(2026,7+1,1)-1))),1)</f>
         <v/>
       </c>
       <c r="N7" s="106">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,8,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,8+1,1))/('📊 ملخص آلي + KPIs'!$F$38*DAY(DATE(2026,8+1,1)-1))),1)</f>
+        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,8,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,8+1,1))/($F$31*DAY(DATE(2026,8+1,1)-1))),1)</f>
         <v/>
       </c>
       <c r="O7" s="106">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,9,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,9+1,1))/('📊 ملخص آلي + KPIs'!$F$38*DAY(DATE(2026,9+1,1)-1))),1)</f>
+        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,9,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,9+1,1))/($F$31*DAY(DATE(2026,9+1,1)-1))),1)</f>
         <v/>
       </c>
       <c r="P7" s="106">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,10,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,10+1,1))/('📊 ملخص آلي + KPIs'!$F$38*DAY(DATE(2026,10+1,1)-1))),1)</f>
+        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,10,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,10+1,1))/($F$31*DAY(DATE(2026,10+1,1)-1))),1)</f>
         <v/>
       </c>
       <c r="Q7" s="106">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,11,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,11+1,1))/('📊 ملخص آلي + KPIs'!$F$38*DAY(DATE(2026,11+1,1)-1))),1)</f>
+        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,11,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,11+1,1))/($F$31*DAY(DATE(2026,11+1,1)-1))),1)</f>
         <v/>
       </c>
       <c r="R7" s="106">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,12,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,12+1,1))/('📊 ملخص آلي + KPIs'!$F$38*DAY(DATE(2026,12+1,1)-1))),1)</f>
+        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,12,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,12+1,1))/($F$31*DAY(DATE(2026,12+1,1)-1))),1)</f>
         <v/>
       </c>
     </row>
@@ -4171,12 +2310,22 @@
     <row r="29">
       <c r="A29" s="83" t="inlineStr">
         <is>
-          <t>ℹ️ المقاييس المطوية متاحة كتشخيص في اللوحة الأصلية: عدد الانقطاعات، دوران المخزون، عدد الحوادث الجسيمة، ونسبة استيفاء الطلبات (Fill Rate).</t>
+          <t>ℹ️ دُمجت ٤ مؤشرات متكررة ضمن هذه التسعة: عدد الانقطاعات←التوفر، الدوران←أيام المخزون، Fill Rate (حُذف)، حوادث النقل←الامتثال/السلامة.</t>
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="117" t="inlineStr">
+        <is>
+          <t>عدد نقاط المنتج (محطات × منتجات) — لحساب «توفر الوقود»</t>
+        </is>
+      </c>
+      <c r="F31" s="118" t="n">
+        <v>300</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="51">
+  <mergeCells count="52">
     <mergeCell ref="A24:A25"/>
     <mergeCell ref="B18:B19"/>
     <mergeCell ref="D21:D22"/>
@@ -4205,6 +2354,7 @@
     <mergeCell ref="A12:E12"/>
     <mergeCell ref="A8:A9"/>
     <mergeCell ref="A29:R29"/>
+    <mergeCell ref="A31:E31"/>
     <mergeCell ref="C8:C9"/>
     <mergeCell ref="D18:D19"/>
     <mergeCell ref="A13:A14"/>
@@ -4244,7 +2394,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4355,7 +2505,7 @@
       </c>
       <c r="H4" s="78" t="inlineStr">
         <is>
-          <t>KPI 1 — حُدِّثت طريقة الحساب</t>
+          <t>K1 — حُدِّثت طريقة الحساب</t>
         </is>
       </c>
     </row>
@@ -4395,7 +2545,7 @@
       </c>
       <c r="H5" s="82" t="inlineStr">
         <is>
-          <t>KPI 6 — حُدِّثت طريقة الحساب</t>
+          <t>K4 — حُدِّثت طريقة الحساب</t>
         </is>
       </c>
     </row>
@@ -4435,7 +2585,7 @@
       </c>
       <c r="H6" s="78" t="inlineStr">
         <is>
-          <t>KPI 8 — مطابقة (دون تغيير)</t>
+          <t>K6 — مطابقة</t>
         </is>
       </c>
     </row>
@@ -4473,7 +2623,7 @@
       </c>
       <c r="H7" s="82" t="inlineStr">
         <is>
-          <t>KPI 3 — مطابقة (دون تغيير)</t>
+          <t>K2 — مطابقة</t>
         </is>
       </c>
     </row>
@@ -4511,7 +2661,7 @@
       </c>
       <c r="H8" s="78" t="inlineStr">
         <is>
-          <t>KPI 4 — مطابقة (دون تغيير)</t>
+          <t>K3 — مطابقة</t>
         </is>
       </c>
     </row>
@@ -4532,7 +2682,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6145,7 +4295,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11968,7 +10118,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19003,7 +17153,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -22932,7 +21082,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Redefine KPIs to measure operational targets directly
Per request, switch 5 KPIs from percentage-achievement to the concrete
operational measure so the displayed target equals the metric's unit:
- توفر الوقود  -> عدد الانقطاعات الشهرية (target 0)
- المواد المخزنية -> متوسط أيام التسليم (<=3); أوامر الشراء -> أيام الإصدار (<=5)
- الامتثال/السلامة -> عدد المخالفات/الحوادث (0); التزام الجدول -> عدد الرحلات المتأخرة (0)
- فواقد/تالفة/مخزون/أسطول unchanged

- Add a zero-target status variant (✅ 0 / 🔴 <annual count>)
- Drop the now-unused product-points input cell
- Update management-reference mapping notes; refresh verify (16 cells) + README

https://claude.ai/code/session_01KvBXTcUzJa33dDsqskcTMw
</commit_message>
<xml_diff>
--- a/workbook/khadija-supply-chain-kpis-2026.xlsx
+++ b/workbook/khadija-supply-chain-kpis-2026.xlsx
@@ -387,7 +387,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="119">
+  <cellXfs count="122">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -741,6 +741,15 @@
     <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="24" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="25" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="22" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1071,7 +1080,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R31"/>
+  <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" style="40" min="1" max="1"/>
@@ -1230,16 +1239,16 @@
       </c>
       <c r="B6" s="102" t="inlineStr">
         <is>
-          <t>توفر الوقود (يطوي عدد الانقطاعات)</t>
+          <t>توفر الوقود — عدد الانقطاعات</t>
         </is>
       </c>
       <c r="C6" s="97" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>انقطاع</t>
         </is>
       </c>
-      <c r="D6" s="115" t="n">
-        <v>0.995</v>
+      <c r="D6" s="119" t="n">
+        <v>0</v>
       </c>
       <c r="E6" s="97" t="inlineStr">
         <is>
@@ -1247,41 +1256,41 @@
         </is>
       </c>
       <c r="F6" s="97" t="n"/>
-      <c r="G6" s="104" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="H6" s="104" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="I6" s="104" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="J6" s="104" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="K6" s="104" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="L6" s="104" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="M6" s="104" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="N6" s="104" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="O6" s="104" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="P6" s="104" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="Q6" s="104" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="R6" s="104" t="n">
-        <v>0.995</v>
+      <c r="G6" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" s="120" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -1291,55 +1300,55 @@
         </is>
       </c>
       <c r="F7" s="105">
-        <f>IFERROR(IF(AVERAGE(G6:R6)=0,"",IF(IFERROR(AVERAGEIF(G7:R7,"&gt;0",G7:R7),0)&gt;=AVERAGE(G6:R6),"✅ ",IF(IFERROR(AVERAGEIF(G7:R7,"&gt;0",G7:R7),0)&gt;=AVERAGE(G6:R6)*0.85,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G7:R7,"&gt;0",G7:R7),0)-AVERAGE(G6:R6))/AVERAGE(G6:R6),"+0.0%;-0.0%")),"")</f>
-        <v/>
-      </c>
-      <c r="G7" s="106">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,1,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,1+1,1))/($F$31*DAY(DATE(2026,1+1,1)-1))),1)</f>
-        <v/>
-      </c>
-      <c r="H7" s="106">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,2,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,2+1,1))/($F$31*DAY(DATE(2026,2+1,1)-1))),1)</f>
-        <v/>
-      </c>
-      <c r="I7" s="106">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,3,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,3+1,1))/($F$31*DAY(DATE(2026,3+1,1)-1))),1)</f>
-        <v/>
-      </c>
-      <c r="J7" s="106">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,4,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,4+1,1))/($F$31*DAY(DATE(2026,4+1,1)-1))),1)</f>
-        <v/>
-      </c>
-      <c r="K7" s="106">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,5,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,5+1,1))/($F$31*DAY(DATE(2026,5+1,1)-1))),1)</f>
-        <v/>
-      </c>
-      <c r="L7" s="106">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,6,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,6+1,1))/($F$31*DAY(DATE(2026,6+1,1)-1))),1)</f>
-        <v/>
-      </c>
-      <c r="M7" s="106">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,7,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,7+1,1))/($F$31*DAY(DATE(2026,7+1,1)-1))),1)</f>
-        <v/>
-      </c>
-      <c r="N7" s="106">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,8,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,8+1,1))/($F$31*DAY(DATE(2026,8+1,1)-1))),1)</f>
-        <v/>
-      </c>
-      <c r="O7" s="106">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,9,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,9+1,1))/($F$31*DAY(DATE(2026,9+1,1)-1))),1)</f>
-        <v/>
-      </c>
-      <c r="P7" s="106">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,10,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,10+1,1))/($F$31*DAY(DATE(2026,10+1,1)-1))),1)</f>
-        <v/>
-      </c>
-      <c r="Q7" s="106">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,11,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,11+1,1))/($F$31*DAY(DATE(2026,11+1,1)-1))),1)</f>
-        <v/>
-      </c>
-      <c r="R7" s="106">
-        <f>IFERROR(1-(SUMIFS('🛢️ انقطاعات الوقود'!F5:F104,'🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,12,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,12+1,1))/($F$31*DAY(DATE(2026,12+1,1)-1))),1)</f>
+        <f>IF(SUM(G7:R7)=0,"✅ 0","🔴 "&amp;TEXT(SUM(G7:R7),"0"))</f>
+        <v/>
+      </c>
+      <c r="G7" s="121">
+        <f>COUNTIFS('🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,1,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,1+1,1))</f>
+        <v/>
+      </c>
+      <c r="H7" s="121">
+        <f>COUNTIFS('🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,2,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,2+1,1))</f>
+        <v/>
+      </c>
+      <c r="I7" s="121">
+        <f>COUNTIFS('🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,3,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,3+1,1))</f>
+        <v/>
+      </c>
+      <c r="J7" s="121">
+        <f>COUNTIFS('🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,4,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,4+1,1))</f>
+        <v/>
+      </c>
+      <c r="K7" s="121">
+        <f>COUNTIFS('🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,5,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,5+1,1))</f>
+        <v/>
+      </c>
+      <c r="L7" s="121">
+        <f>COUNTIFS('🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,6,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,6+1,1))</f>
+        <v/>
+      </c>
+      <c r="M7" s="121">
+        <f>COUNTIFS('🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,7,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,7+1,1))</f>
+        <v/>
+      </c>
+      <c r="N7" s="121">
+        <f>COUNTIFS('🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,8,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,8+1,1))</f>
+        <v/>
+      </c>
+      <c r="O7" s="121">
+        <f>COUNTIFS('🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,9,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,9+1,1))</f>
+        <v/>
+      </c>
+      <c r="P7" s="121">
+        <f>COUNTIFS('🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,10,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,10+1,1))</f>
+        <v/>
+      </c>
+      <c r="Q7" s="121">
+        <f>COUNTIFS('🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,11,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,11+1,1))</f>
+        <v/>
+      </c>
+      <c r="R7" s="121">
+        <f>COUNTIFS('🛢️ انقطاعات الوقود'!B5:B104,"&gt;="&amp;DATE(2026,12,1),'🛢️ انقطاعات الوقود'!B5:B104,"&lt;"&amp;DATE(2026,12+1,1))</f>
         <v/>
       </c>
     </row>
@@ -1349,16 +1358,16 @@
       </c>
       <c r="B8" s="102" t="inlineStr">
         <is>
-          <t>توفر المواد المخزنية (تسليم ≤ 3 أيام)</t>
+          <t>توفر المواد المخزنية — أيام التسليم</t>
         </is>
       </c>
       <c r="C8" s="97" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>يوم</t>
         </is>
       </c>
-      <c r="D8" s="115" t="n">
-        <v>1</v>
+      <c r="D8" s="116" t="n">
+        <v>3</v>
       </c>
       <c r="E8" s="97" t="inlineStr">
         <is>
@@ -1366,41 +1375,41 @@
         </is>
       </c>
       <c r="F8" s="97" t="n"/>
-      <c r="G8" s="104" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" s="104" t="n">
-        <v>1</v>
-      </c>
-      <c r="I8" s="104" t="n">
-        <v>1</v>
-      </c>
-      <c r="J8" s="104" t="n">
-        <v>1</v>
-      </c>
-      <c r="K8" s="104" t="n">
-        <v>1</v>
-      </c>
-      <c r="L8" s="104" t="n">
-        <v>1</v>
-      </c>
-      <c r="M8" s="104" t="n">
-        <v>1</v>
-      </c>
-      <c r="N8" s="104" t="n">
-        <v>1</v>
-      </c>
-      <c r="O8" s="104" t="n">
-        <v>1</v>
-      </c>
-      <c r="P8" s="104" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q8" s="104" t="n">
-        <v>1</v>
-      </c>
-      <c r="R8" s="104" t="n">
-        <v>1</v>
+      <c r="G8" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="I8" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="J8" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="K8" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="L8" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="M8" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="N8" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="O8" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="P8" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q8" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="R8" s="107" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -1410,55 +1419,55 @@
         </is>
       </c>
       <c r="F9" s="105">
-        <f>IFERROR(IF(AVERAGE(G8:R8)=0,"",IF(IFERROR(AVERAGEIF(G9:R9,"&gt;0",G9:R9),0)&gt;=AVERAGE(G8:R8),"✅ ",IF(IFERROR(AVERAGEIF(G9:R9,"&gt;0",G9:R9),0)&gt;=AVERAGE(G8:R8)*0.85,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G9:R9,"&gt;0",G9:R9),0)-AVERAGE(G8:R8))/AVERAGE(G8:R8),"+0.0%;-0.0%")),"")</f>
-        <v/>
-      </c>
-      <c r="G9" s="106">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,1,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,1+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,1,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,1+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
-        <v/>
-      </c>
-      <c r="H9" s="106">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,2,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,2+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,2,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,2+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
-        <v/>
-      </c>
-      <c r="I9" s="106">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,3,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,3+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,3,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,3+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
-        <v/>
-      </c>
-      <c r="J9" s="106">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,4,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,4+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,4,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,4+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
-        <v/>
-      </c>
-      <c r="K9" s="106">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,5,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,5+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,5,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,5+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
-        <v/>
-      </c>
-      <c r="L9" s="106">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,6,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,6+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,6,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,6+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
-        <v/>
-      </c>
-      <c r="M9" s="106">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,7,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,7+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,7,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,7+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
-        <v/>
-      </c>
-      <c r="N9" s="106">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,8,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,8+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,8,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,8+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
-        <v/>
-      </c>
-      <c r="O9" s="106">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,9,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,9+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,9,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,9+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
-        <v/>
-      </c>
-      <c r="P9" s="106">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,10,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,10+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,10,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,10+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
-        <v/>
-      </c>
-      <c r="Q9" s="106">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,11,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,11+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,11,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,11+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
-        <v/>
-      </c>
-      <c r="R9" s="106">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,12,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,12+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,12,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,12+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية")),0)</f>
+        <f>IFERROR(IF(AVERAGE(G8:R8)=0,"",IF(IFERROR(AVERAGEIF(G9:R9,"&gt;0",G9:R9),0)&lt;=AVERAGE(G8:R8),"✅ ",IF(IFERROR(AVERAGEIF(G9:R9,"&gt;0",G9:R9),0)&lt;=AVERAGE(G8:R8)*1.3,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G9:R9,"&gt;0",G9:R9),0)-AVERAGE(G8:R8))/AVERAGE(G8:R8),"+0.0%;-0.0%")),"")</f>
+        <v/>
+      </c>
+      <c r="G9" s="108">
+        <f>IFERROR(AVERAGEIFS('🛒 الطلبات والمشتريات'!H5:H204,'🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,1,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,1+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية"),0)</f>
+        <v/>
+      </c>
+      <c r="H9" s="108">
+        <f>IFERROR(AVERAGEIFS('🛒 الطلبات والمشتريات'!H5:H204,'🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,2,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,2+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية"),0)</f>
+        <v/>
+      </c>
+      <c r="I9" s="108">
+        <f>IFERROR(AVERAGEIFS('🛒 الطلبات والمشتريات'!H5:H204,'🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,3,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,3+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية"),0)</f>
+        <v/>
+      </c>
+      <c r="J9" s="108">
+        <f>IFERROR(AVERAGEIFS('🛒 الطلبات والمشتريات'!H5:H204,'🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,4,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,4+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية"),0)</f>
+        <v/>
+      </c>
+      <c r="K9" s="108">
+        <f>IFERROR(AVERAGEIFS('🛒 الطلبات والمشتريات'!H5:H204,'🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,5,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,5+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية"),0)</f>
+        <v/>
+      </c>
+      <c r="L9" s="108">
+        <f>IFERROR(AVERAGEIFS('🛒 الطلبات والمشتريات'!H5:H204,'🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,6,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,6+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية"),0)</f>
+        <v/>
+      </c>
+      <c r="M9" s="108">
+        <f>IFERROR(AVERAGEIFS('🛒 الطلبات والمشتريات'!H5:H204,'🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,7,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,7+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية"),0)</f>
+        <v/>
+      </c>
+      <c r="N9" s="108">
+        <f>IFERROR(AVERAGEIFS('🛒 الطلبات والمشتريات'!H5:H204,'🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,8,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,8+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية"),0)</f>
+        <v/>
+      </c>
+      <c r="O9" s="108">
+        <f>IFERROR(AVERAGEIFS('🛒 الطلبات والمشتريات'!H5:H204,'🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,9,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,9+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية"),0)</f>
+        <v/>
+      </c>
+      <c r="P9" s="108">
+        <f>IFERROR(AVERAGEIFS('🛒 الطلبات والمشتريات'!H5:H204,'🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,10,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,10+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية"),0)</f>
+        <v/>
+      </c>
+      <c r="Q9" s="108">
+        <f>IFERROR(AVERAGEIFS('🛒 الطلبات والمشتريات'!H5:H204,'🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,11,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,11+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية"),0)</f>
+        <v/>
+      </c>
+      <c r="R9" s="108">
+        <f>IFERROR(AVERAGEIFS('🛒 الطلبات والمشتريات'!H5:H204,'🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,12,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,12+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"مواد مخزنية"),0)</f>
         <v/>
       </c>
     </row>
@@ -1468,16 +1477,16 @@
       </c>
       <c r="B10" s="102" t="inlineStr">
         <is>
-          <t>إصدار أوامر الشراء (≤ 5 أيام عمل)</t>
+          <t>إصدار أوامر الشراء — أيام الإصدار</t>
         </is>
       </c>
       <c r="C10" s="97" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>يوم</t>
         </is>
       </c>
-      <c r="D10" s="115" t="n">
-        <v>0.95</v>
+      <c r="D10" s="116" t="n">
+        <v>5</v>
       </c>
       <c r="E10" s="97" t="inlineStr">
         <is>
@@ -1485,41 +1494,41 @@
         </is>
       </c>
       <c r="F10" s="97" t="n"/>
-      <c r="G10" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="H10" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="I10" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="J10" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="K10" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="L10" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="M10" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="N10" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="O10" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="P10" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="Q10" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="R10" s="104" t="n">
-        <v>0.95</v>
+      <c r="G10" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="H10" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="I10" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="J10" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="K10" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="L10" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="M10" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="N10" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="O10" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="P10" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q10" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="R10" s="107" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="11">
@@ -1529,55 +1538,55 @@
         </is>
       </c>
       <c r="F11" s="105">
-        <f>IFERROR(IF(AVERAGE(G10:R10)=0,"",IF(IFERROR(AVERAGEIF(G11:R11,"&gt;0",G11:R11),0)&gt;=AVERAGE(G10:R10),"✅ ",IF(IFERROR(AVERAGEIF(G11:R11,"&gt;0",G11:R11),0)&gt;=AVERAGE(G10:R10)*0.85,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G11:R11,"&gt;0",G11:R11),0)-AVERAGE(G10:R10))/AVERAGE(G10:R10),"+0.0%;-0.0%")),"")</f>
-        <v/>
-      </c>
-      <c r="G11" s="106">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,1,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,1+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,1,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,1+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
-        <v/>
-      </c>
-      <c r="H11" s="106">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,2,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,2+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,2,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,2+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
-        <v/>
-      </c>
-      <c r="I11" s="106">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,3,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,3+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,3,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,3+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
-        <v/>
-      </c>
-      <c r="J11" s="106">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,4,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,4+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,4,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,4+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
-        <v/>
-      </c>
-      <c r="K11" s="106">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,5,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,5+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,5,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,5+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
-        <v/>
-      </c>
-      <c r="L11" s="106">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,6,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,6+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,6,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,6+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
-        <v/>
-      </c>
-      <c r="M11" s="106">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,7,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,7+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,7,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,7+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
-        <v/>
-      </c>
-      <c r="N11" s="106">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,8,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,8+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,8,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,8+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
-        <v/>
-      </c>
-      <c r="O11" s="106">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,9,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,9+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,9,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,9+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
-        <v/>
-      </c>
-      <c r="P11" s="106">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,10,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,10+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,10,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,10+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
-        <v/>
-      </c>
-      <c r="Q11" s="106">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,11,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,11+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,11,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,11+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
-        <v/>
-      </c>
-      <c r="R11" s="106">
-        <f>IFERROR(COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,12,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,12+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء",'🛒 الطلبات والمشتريات'!I5:I204,"*ضمن*")/MAX(1,COUNTIFS('🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,12,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,12+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء")),0)</f>
+        <f>IFERROR(IF(AVERAGE(G10:R10)=0,"",IF(IFERROR(AVERAGEIF(G11:R11,"&gt;0",G11:R11),0)&lt;=AVERAGE(G10:R10),"✅ ",IF(IFERROR(AVERAGEIF(G11:R11,"&gt;0",G11:R11),0)&lt;=AVERAGE(G10:R10)*1.3,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G11:R11,"&gt;0",G11:R11),0)-AVERAGE(G10:R10))/AVERAGE(G10:R10),"+0.0%;-0.0%")),"")</f>
+        <v/>
+      </c>
+      <c r="G11" s="108">
+        <f>IFERROR(AVERAGEIFS('🛒 الطلبات والمشتريات'!H5:H204,'🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,1,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,1+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء"),0)</f>
+        <v/>
+      </c>
+      <c r="H11" s="108">
+        <f>IFERROR(AVERAGEIFS('🛒 الطلبات والمشتريات'!H5:H204,'🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,2,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,2+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء"),0)</f>
+        <v/>
+      </c>
+      <c r="I11" s="108">
+        <f>IFERROR(AVERAGEIFS('🛒 الطلبات والمشتريات'!H5:H204,'🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,3,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,3+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء"),0)</f>
+        <v/>
+      </c>
+      <c r="J11" s="108">
+        <f>IFERROR(AVERAGEIFS('🛒 الطلبات والمشتريات'!H5:H204,'🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,4,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,4+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء"),0)</f>
+        <v/>
+      </c>
+      <c r="K11" s="108">
+        <f>IFERROR(AVERAGEIFS('🛒 الطلبات والمشتريات'!H5:H204,'🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,5,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,5+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء"),0)</f>
+        <v/>
+      </c>
+      <c r="L11" s="108">
+        <f>IFERROR(AVERAGEIFS('🛒 الطلبات والمشتريات'!H5:H204,'🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,6,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,6+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء"),0)</f>
+        <v/>
+      </c>
+      <c r="M11" s="108">
+        <f>IFERROR(AVERAGEIFS('🛒 الطلبات والمشتريات'!H5:H204,'🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,7,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,7+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء"),0)</f>
+        <v/>
+      </c>
+      <c r="N11" s="108">
+        <f>IFERROR(AVERAGEIFS('🛒 الطلبات والمشتريات'!H5:H204,'🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,8,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,8+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء"),0)</f>
+        <v/>
+      </c>
+      <c r="O11" s="108">
+        <f>IFERROR(AVERAGEIFS('🛒 الطلبات والمشتريات'!H5:H204,'🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,9,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,9+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء"),0)</f>
+        <v/>
+      </c>
+      <c r="P11" s="108">
+        <f>IFERROR(AVERAGEIFS('🛒 الطلبات والمشتريات'!H5:H204,'🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,10,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,10+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء"),0)</f>
+        <v/>
+      </c>
+      <c r="Q11" s="108">
+        <f>IFERROR(AVERAGEIFS('🛒 الطلبات والمشتريات'!H5:H204,'🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,11,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,11+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء"),0)</f>
+        <v/>
+      </c>
+      <c r="R11" s="108">
+        <f>IFERROR(AVERAGEIFS('🛒 الطلبات والمشتريات'!H5:H204,'🛒 الطلبات والمشتريات'!C5:C204,"&gt;="&amp;DATE(2026,12,1),'🛒 الطلبات والمشتريات'!C5:C204,"&lt;"&amp;DATE(2026,12+1,1),'🛒 الطلبات والمشتريات'!D5:D204,"أمر شراء"),0)</f>
         <v/>
       </c>
     </row>
@@ -1813,7 +1822,7 @@
       </c>
       <c r="B18" s="102" t="inlineStr">
         <is>
-          <t>أيام مخزون الوقود (يطوي الدوران)</t>
+          <t>أيام مخزون الوقود</t>
         </is>
       </c>
       <c r="C18" s="97" t="inlineStr">
@@ -1944,16 +1953,16 @@
       </c>
       <c r="B21" s="102" t="inlineStr">
         <is>
-          <t>الامتثال والسلامة (يطوي عدد الحوادث)</t>
+          <t>الامتثال والسلامة — المخالفات/الحوادث</t>
         </is>
       </c>
       <c r="C21" s="97" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>مخالفة</t>
         </is>
       </c>
-      <c r="D21" s="115" t="n">
-        <v>0.95</v>
+      <c r="D21" s="119" t="n">
+        <v>0</v>
       </c>
       <c r="E21" s="97" t="inlineStr">
         <is>
@@ -1961,41 +1970,41 @@
         </is>
       </c>
       <c r="F21" s="97" t="n"/>
-      <c r="G21" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="H21" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="I21" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="J21" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="K21" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="L21" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="M21" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="N21" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="O21" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="P21" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="Q21" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="R21" s="104" t="n">
-        <v>0.95</v>
+      <c r="G21" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" s="120" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -2005,55 +2014,55 @@
         </is>
       </c>
       <c r="F22" s="105">
-        <f>IFERROR(IF(AVERAGE(G21:R21)=0,"",IF(IFERROR(AVERAGEIF(G22:R22,"&gt;0",G22:R22),0)&gt;=AVERAGE(G21:R21),"✅ ",IF(IFERROR(AVERAGEIF(G22:R22,"&gt;0",G22:R22),0)&gt;=AVERAGE(G21:R21)*0.85,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G22:R22,"&gt;0",G22:R22),0)-AVERAGE(G21:R21))/AVERAGE(G21:R21),"+0.0%;-0.0%")),"")</f>
-        <v/>
-      </c>
-      <c r="G22" s="106">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,1,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,1+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,1,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,1+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="H22" s="106">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,2,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,2+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,2,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,2+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="I22" s="106">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,3,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,3+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,3,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,3+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="J22" s="106">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,4,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,4+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,4,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,4+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="K22" s="106">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,5,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,5+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,5,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,5+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="L22" s="106">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,6,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,6+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,6,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,6+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="M22" s="106">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,7,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,7+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,7,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,7+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="N22" s="106">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,8,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,8+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,8,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,8+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="O22" s="106">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,9,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,9+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,9,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,9+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="P22" s="106">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,10,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,10+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,10,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,10+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="Q22" s="106">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,11,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,11+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,11,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,11+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="R22" s="106">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,12,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,12+1,1),'🚚 النقل والرحلات'!K5:K304,"لا يوجد")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,12,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,12+1,1))),0)</f>
+        <f>IF(SUM(G22:R22)=0,"✅ 0","🔴 "&amp;TEXT(SUM(G22:R22),"0"))</f>
+        <v/>
+      </c>
+      <c r="G22" s="121">
+        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,1,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,1+1,1),'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;لا يوجد",'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="H22" s="121">
+        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,2,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,2+1,1),'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;لا يوجد",'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="I22" s="121">
+        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,3,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,3+1,1),'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;لا يوجد",'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="J22" s="121">
+        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,4,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,4+1,1),'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;لا يوجد",'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="K22" s="121">
+        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,5,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,5+1,1),'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;لا يوجد",'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="L22" s="121">
+        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,6,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,6+1,1),'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;لا يوجد",'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="M22" s="121">
+        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,7,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,7+1,1),'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;لا يوجد",'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="N22" s="121">
+        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,8,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,8+1,1),'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;لا يوجد",'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="O22" s="121">
+        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,9,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,9+1,1),'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;لا يوجد",'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="P22" s="121">
+        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,10,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,10+1,1),'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;لا يوجد",'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="Q22" s="121">
+        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,11,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,11+1,1),'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;لا يوجد",'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="R22" s="121">
+        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,12,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,12+1,1),'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;لا يوجد",'🚚 النقل والرحلات'!K5:K304,"&lt;&gt;")</f>
         <v/>
       </c>
     </row>
@@ -2075,16 +2084,16 @@
       </c>
       <c r="B24" s="102" t="inlineStr">
         <is>
-          <t>التزام جدول النقل (On-time)</t>
+          <t>التزام جدول النقل — الرحلات المتأخرة</t>
         </is>
       </c>
       <c r="C24" s="97" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>رحلة</t>
         </is>
       </c>
-      <c r="D24" s="115" t="n">
-        <v>0.95</v>
+      <c r="D24" s="119" t="n">
+        <v>0</v>
       </c>
       <c r="E24" s="97" t="inlineStr">
         <is>
@@ -2092,41 +2101,41 @@
         </is>
       </c>
       <c r="F24" s="97" t="n"/>
-      <c r="G24" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="H24" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="I24" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="J24" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="K24" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="L24" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="M24" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="N24" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="O24" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="P24" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="Q24" s="104" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="R24" s="104" t="n">
-        <v>0.95</v>
+      <c r="G24" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="R24" s="120" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -2136,55 +2145,55 @@
         </is>
       </c>
       <c r="F25" s="105">
-        <f>IFERROR(IF(AVERAGE(G24:R24)=0,"",IF(IFERROR(AVERAGEIF(G25:R25,"&gt;0",G25:R25),0)&gt;=AVERAGE(G24:R24),"✅ ",IF(IFERROR(AVERAGEIF(G25:R25,"&gt;0",G25:R25),0)&gt;=AVERAGE(G24:R24)*0.85,"🟡 ","🔴 "))&amp;TEXT((IFERROR(AVERAGEIF(G25:R25,"&gt;0",G25:R25),0)-AVERAGE(G24:R24))/AVERAGE(G24:R24),"+0.0%;-0.0%")),"")</f>
-        <v/>
-      </c>
-      <c r="G25" s="106">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,1,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,1+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,1,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,1+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="H25" s="106">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,2,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,2+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,2,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,2+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="I25" s="106">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,3,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,3+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,3,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,3+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="J25" s="106">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,4,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,4+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,4,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,4+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="K25" s="106">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,5,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,5+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,5,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,5+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="L25" s="106">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,6,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,6+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,6,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,6+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="M25" s="106">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,7,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,7+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,7,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,7+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="N25" s="106">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,8,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,8+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,8,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,8+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="O25" s="106">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,9,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,9+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,9,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,9+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="P25" s="106">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,10,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,10+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,10,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,10+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="Q25" s="106">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,11,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,11+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,11,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,11+1,1))),0)</f>
-        <v/>
-      </c>
-      <c r="R25" s="106">
-        <f>IFERROR(COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,12,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,12+1,1),'🚚 النقل والرحلات'!J5:J304,"*في الوقت*")/MAX(1,COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,12,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,12+1,1))),0)</f>
+        <f>IF(SUM(G25:R25)=0,"✅ 0","🔴 "&amp;TEXT(SUM(G25:R25),"0"))</f>
+        <v/>
+      </c>
+      <c r="G25" s="121">
+        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,1,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,1+1,1),'🚚 النقل والرحلات'!J5:J304,"*متأخر*")</f>
+        <v/>
+      </c>
+      <c r="H25" s="121">
+        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,2,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,2+1,1),'🚚 النقل والرحلات'!J5:J304,"*متأخر*")</f>
+        <v/>
+      </c>
+      <c r="I25" s="121">
+        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,3,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,3+1,1),'🚚 النقل والرحلات'!J5:J304,"*متأخر*")</f>
+        <v/>
+      </c>
+      <c r="J25" s="121">
+        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,4,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,4+1,1),'🚚 النقل والرحلات'!J5:J304,"*متأخر*")</f>
+        <v/>
+      </c>
+      <c r="K25" s="121">
+        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,5,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,5+1,1),'🚚 النقل والرحلات'!J5:J304,"*متأخر*")</f>
+        <v/>
+      </c>
+      <c r="L25" s="121">
+        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,6,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,6+1,1),'🚚 النقل والرحلات'!J5:J304,"*متأخر*")</f>
+        <v/>
+      </c>
+      <c r="M25" s="121">
+        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,7,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,7+1,1),'🚚 النقل والرحلات'!J5:J304,"*متأخر*")</f>
+        <v/>
+      </c>
+      <c r="N25" s="121">
+        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,8,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,8+1,1),'🚚 النقل والرحلات'!J5:J304,"*متأخر*")</f>
+        <v/>
+      </c>
+      <c r="O25" s="121">
+        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,9,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,9+1,1),'🚚 النقل والرحلات'!J5:J304,"*متأخر*")</f>
+        <v/>
+      </c>
+      <c r="P25" s="121">
+        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,10,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,10+1,1),'🚚 النقل والرحلات'!J5:J304,"*متأخر*")</f>
+        <v/>
+      </c>
+      <c r="Q25" s="121">
+        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,11,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,11+1,1),'🚚 النقل والرحلات'!J5:J304,"*متأخر*")</f>
+        <v/>
+      </c>
+      <c r="R25" s="121">
+        <f>COUNTIFS('🚚 النقل والرحلات'!B5:B304,"&gt;="&amp;DATE(2026,12,1),'🚚 النقل والرحلات'!B5:B304,"&lt;"&amp;DATE(2026,12+1,1),'🚚 النقل والرحلات'!J5:J304,"*متأخر*")</f>
         <v/>
       </c>
     </row>
@@ -2310,22 +2319,12 @@
     <row r="29">
       <c r="A29" s="83" t="inlineStr">
         <is>
-          <t>ℹ️ دُمجت ٤ مؤشرات متكررة ضمن هذه التسعة: عدد الانقطاعات←التوفر، الدوران←أيام المخزون، Fill Rate (حُذف)، حوادث النقل←الامتثال/السلامة.</t>
+          <t>ℹ️ أهداف تشغيلية: الانقطاعات/المخالفات/المتأخرات هدفها 0 ، وأيام التسليم/الإصدار/المخزون حدّها أعلى. دُمجت ٤ مؤشرات متكررة في هذه التسعة.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="117" t="inlineStr">
-        <is>
-          <t>عدد نقاط المنتج (محطات × منتجات) — لحساب «توفر الوقود»</t>
-        </is>
-      </c>
-      <c r="F31" s="118" t="n">
-        <v>300</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="52">
+  <mergeCells count="51">
     <mergeCell ref="A24:A25"/>
     <mergeCell ref="B18:B19"/>
     <mergeCell ref="D21:D22"/>
@@ -2354,7 +2353,6 @@
     <mergeCell ref="A12:E12"/>
     <mergeCell ref="A8:A9"/>
     <mergeCell ref="A29:R29"/>
-    <mergeCell ref="A31:E31"/>
     <mergeCell ref="C8:C9"/>
     <mergeCell ref="D18:D19"/>
     <mergeCell ref="A13:A14"/>
@@ -2505,7 +2503,7 @@
       </c>
       <c r="H4" s="78" t="inlineStr">
         <is>
-          <t>K1 — حُدِّثت طريقة الحساب</t>
+          <t>K1 — عدد الانقطاعات (هدف 0)</t>
         </is>
       </c>
     </row>
@@ -2623,7 +2621,7 @@
       </c>
       <c r="H7" s="82" t="inlineStr">
         <is>
-          <t>K2 — مطابقة</t>
+          <t>K2 — أيام التسليم (≤3)</t>
         </is>
       </c>
     </row>
@@ -2661,7 +2659,7 @@
       </c>
       <c r="H8" s="78" t="inlineStr">
         <is>
-          <t>K3 — مطابقة</t>
+          <t>K3 — أيام الإصدار (≤5)</t>
         </is>
       </c>
     </row>

</xml_diff>